<commit_message>
Mahal listesi ve ağırlık cetveli güncellendi (MAHAL-AGIRLIK-EKSIKSIZ)
</commit_message>
<xml_diff>
--- a/belgeler/03_METRAJ_CETVELI.xlsx
+++ b/belgeler/03_METRAJ_CETVELI.xlsx
@@ -186,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -280,6 +280,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -10539,7 +10542,7 @@
       <c r="B406" s="6" t="n"/>
       <c r="C406" s="23" t="inlineStr">
         <is>
-          <t>Foseptik — betonarme gövdenin iç hacmi 1.50x1.50x2.50 = 5.62 m³; en yakın standart tank 6 m³</t>
+          <t>Foseptik — kazı çukurunun net oturma alanına sığan hazne 1.50x1.50x2.50 = 5.62 m³; en yakın standart tank 6 m³</t>
         </is>
       </c>
       <c r="D406" s="6" t="n"/>
@@ -13513,15 +13516,15 @@
           <t>AÇIKLAMALAR</t>
         </is>
       </c>
-      <c r="B529" s="39" t="n"/>
-      <c r="C529" s="39" t="n"/>
-      <c r="D529" s="39" t="n"/>
-      <c r="E529" s="39" t="n"/>
-      <c r="F529" s="39" t="n"/>
-      <c r="G529" s="39" t="n"/>
-      <c r="H529" s="39" t="n"/>
-      <c r="I529" s="39" t="n"/>
-      <c r="J529" s="40" t="n"/>
+      <c r="B529" s="40" t="n"/>
+      <c r="C529" s="40" t="n"/>
+      <c r="D529" s="40" t="n"/>
+      <c r="E529" s="40" t="n"/>
+      <c r="F529" s="40" t="n"/>
+      <c r="G529" s="40" t="n"/>
+      <c r="H529" s="40" t="n"/>
+      <c r="I529" s="40" t="n"/>
+      <c r="J529" s="41" t="n"/>
     </row>
     <row r="530" ht="13" customHeight="1">
       <c r="A530" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Yayın: yem silosu kaideleri onaylı statik projeye göre metrajlandı (SILO-KAIDE-PROJESI)
Radye 2,90x2,90x0,40 + SB01…SB04 kolonları 40/40x1,10. Metraj yenilendi,
proforma ve A3.4-EK 72.659,08 TL ile ekranla aynı kaldı.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/03_METRAJ_CETVELI.xlsx
+++ b/belgeler/03_METRAJ_CETVELI.xlsx
@@ -652,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J551"/>
+  <dimension ref="A1:J556"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11168,12 +11168,12 @@
       <c r="I429" s="22" t="n"/>
       <c r="J429" s="22" t="n"/>
     </row>
-    <row r="430" ht="20" customHeight="1">
+    <row r="430" ht="30" customHeight="1">
       <c r="A430" s="6" t="n"/>
       <c r="B430" s="6" t="n"/>
       <c r="C430" s="23" t="inlineStr">
         <is>
-          <t>Silo kaideleri: 2.90x2.90 kaide; 1,00 m çalışma payı -&gt; 4.90x4.90; derinlik 1,00 m</t>
+          <t>Silo kaideleri: radye 2,90x2,90; 0,50 m çalışma payı -&gt; 3,90x3,90; radye altı -0,10 + 10 cm grobeton = 0,20 m derinlik</t>
         </is>
       </c>
       <c r="D430" s="6" t="n"/>
@@ -11181,13 +11181,13 @@
         <v>2</v>
       </c>
       <c r="F430" s="29" t="n">
-        <v>4.9</v>
+        <v>3.9</v>
       </c>
       <c r="G430" s="29" t="n">
-        <v>4.9</v>
+        <v>3.9</v>
       </c>
       <c r="H430" s="29" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I430" s="24">
         <f>E430*F430*G430*H430</f>
@@ -11320,12 +11320,12 @@
       <c r="I435" s="22" t="n"/>
       <c r="J435" s="22" t="n"/>
     </row>
-    <row r="436" ht="12" customHeight="1">
+    <row r="436" ht="20" customHeight="1">
       <c r="A436" s="6" t="n"/>
       <c r="B436" s="6" t="n"/>
       <c r="C436" s="23" t="inlineStr">
         <is>
-          <t>Silo betonarme kaidesi (2 adet)</t>
+          <t>Radye temel 2,90x2,90, H = 0,40 m (-0,10 / +0,30); 2 kaide — proje METRAJ tablosu 3,36 m³/kaide</t>
         </is>
       </c>
       <c r="D436" s="6" t="n"/>
@@ -11339,7 +11339,7 @@
         <v>2.9</v>
       </c>
       <c r="H436" s="29" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="I436" s="24">
         <f>E436*F436*G436*H436</f>
@@ -11347,46 +11347,44 @@
       </c>
       <c r="J436" s="6" t="n"/>
     </row>
-    <row r="437">
-      <c r="A437" s="22" t="n"/>
-      <c r="B437" s="22" t="n"/>
-      <c r="C437" s="25" t="inlineStr">
+    <row r="437" ht="30" customHeight="1">
+      <c r="A437" s="6" t="n"/>
+      <c r="B437" s="6" t="n"/>
+      <c r="C437" s="23" t="inlineStr">
+        <is>
+          <t>SB01…SB04 bodrum kat kolonları 40/40 (+0,30 / +1,40): 4 ad x 2 kaide, yükseklik 1,10 m — proje METRAJ tablosu 0,70 m³/kaide</t>
+        </is>
+      </c>
+      <c r="D437" s="6" t="n"/>
+      <c r="E437" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="F437" s="29" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G437" s="29" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H437" s="29" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I437" s="24">
+        <f>E437*F437*G437*H437</f>
+        <v/>
+      </c>
+      <c r="J437" s="6" t="n"/>
+    </row>
+    <row r="438">
+      <c r="A438" s="22" t="n"/>
+      <c r="B438" s="22" t="n"/>
+      <c r="C438" s="25" t="inlineStr">
         <is>
           <t>M17 TOPLAMI</t>
         </is>
       </c>
-      <c r="D437" s="26" t="inlineStr">
+      <c r="D438" s="26" t="inlineStr">
         <is>
           <t>m³</t>
-        </is>
-      </c>
-      <c r="E437" s="22" t="n"/>
-      <c r="F437" s="22" t="n"/>
-      <c r="G437" s="22" t="n"/>
-      <c r="H437" s="22" t="n"/>
-      <c r="I437" s="22" t="n"/>
-      <c r="J437" s="27">
-        <f>SUM(I436:I436)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="438" ht="15" customHeight="1">
-      <c r="A438" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="B438" s="20" t="inlineStr">
-        <is>
-          <t>15.180.1003</t>
-        </is>
-      </c>
-      <c r="C438" s="8" t="inlineStr">
-        <is>
-          <t>[M21]  Plywood ile düz yüzeyli betonarme kalıbı — silo kaideleri</t>
-        </is>
-      </c>
-      <c r="D438" s="21" t="inlineStr">
-        <is>
-          <t>m²</t>
         </is>
       </c>
       <c r="E438" s="22" t="n"/>
@@ -11394,120 +11392,125 @@
       <c r="G438" s="22" t="n"/>
       <c r="H438" s="22" t="n"/>
       <c r="I438" s="22" t="n"/>
-      <c r="J438" s="22" t="n"/>
-    </row>
-    <row r="439" ht="20" customHeight="1">
-      <c r="A439" s="6" t="n"/>
-      <c r="B439" s="6" t="n"/>
-      <c r="C439" s="23" t="inlineStr">
-        <is>
-          <t>Silo kaidesi yan yüzleri: 4 yüz x 2 adet, boy 2.90, yükseklik 0.50</t>
-        </is>
-      </c>
-      <c r="D439" s="6" t="n"/>
-      <c r="E439" s="28" t="n">
+      <c r="J438" s="27">
+        <f>SUM(I436:I437)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="439" ht="15" customHeight="1">
+      <c r="A439" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="B439" s="20" t="inlineStr">
+        <is>
+          <t>15.180.1003</t>
+        </is>
+      </c>
+      <c r="C439" s="8" t="inlineStr">
+        <is>
+          <t>[M21]  Plywood ile düz yüzeyli betonarme kalıbı — silo kaideleri</t>
+        </is>
+      </c>
+      <c r="D439" s="21" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E439" s="22" t="n"/>
+      <c r="F439" s="22" t="n"/>
+      <c r="G439" s="22" t="n"/>
+      <c r="H439" s="22" t="n"/>
+      <c r="I439" s="22" t="n"/>
+      <c r="J439" s="22" t="n"/>
+    </row>
+    <row r="440" ht="20" customHeight="1">
+      <c r="A440" s="6" t="n"/>
+      <c r="B440" s="6" t="n"/>
+      <c r="C440" s="23" t="inlineStr">
+        <is>
+          <t>Radye temel yan yüzleri: 4 yüz x 2 kaide, boy 2,90 m, yükseklik 0,40 m — proje METRAJ tablosu 4,64 m²/kaide</t>
+        </is>
+      </c>
+      <c r="D440" s="6" t="n"/>
+      <c r="E440" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="F439" s="6" t="n"/>
-      <c r="G439" s="29" t="n">
+      <c r="F440" s="6" t="n"/>
+      <c r="G440" s="29" t="n">
         <v>2.9</v>
       </c>
-      <c r="H439" s="29" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I439" s="24">
-        <f>E439*G439*H439</f>
-        <v/>
-      </c>
-      <c r="J439" s="6" t="n"/>
-    </row>
-    <row r="440">
-      <c r="A440" s="22" t="n"/>
-      <c r="B440" s="22" t="n"/>
-      <c r="C440" s="25" t="inlineStr">
+      <c r="H440" s="29" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I440" s="24">
+        <f>E440*G440*H440</f>
+        <v/>
+      </c>
+      <c r="J440" s="6" t="n"/>
+    </row>
+    <row r="441" ht="30" customHeight="1">
+      <c r="A441" s="6" t="n"/>
+      <c r="B441" s="6" t="n"/>
+      <c r="C441" s="23" t="inlineStr">
+        <is>
+          <t>SB01…SB04 kolon yüzleri: 4 kolon x 4 yüz x 2 kaide = 32; genişlik 0,40 m, yükseklik 1,10 m — proje METRAJ tablosu 7,04 m²/kaide</t>
+        </is>
+      </c>
+      <c r="D441" s="6" t="n"/>
+      <c r="E441" s="28" t="n">
+        <v>32</v>
+      </c>
+      <c r="F441" s="6" t="n"/>
+      <c r="G441" s="29" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H441" s="29" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I441" s="24">
+        <f>E441*G441*H441</f>
+        <v/>
+      </c>
+      <c r="J441" s="6" t="n"/>
+    </row>
+    <row r="442">
+      <c r="A442" s="22" t="n"/>
+      <c r="B442" s="22" t="n"/>
+      <c r="C442" s="25" t="inlineStr">
         <is>
           <t>M21 TOPLAMI</t>
         </is>
       </c>
-      <c r="D440" s="26" t="inlineStr">
+      <c r="D442" s="26" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E440" s="22" t="n"/>
-      <c r="F440" s="22" t="n"/>
-      <c r="G440" s="22" t="n"/>
-      <c r="H440" s="22" t="n"/>
-      <c r="I440" s="22" t="n"/>
-      <c r="J440" s="27">
-        <f>SUM(I439:I439)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="441" ht="22" customHeight="1">
-      <c r="A441" s="19" t="n">
+      <c r="E442" s="22" t="n"/>
+      <c r="F442" s="22" t="n"/>
+      <c r="G442" s="22" t="n"/>
+      <c r="H442" s="22" t="n"/>
+      <c r="I442" s="22" t="n"/>
+      <c r="J442" s="27">
+        <f>SUM(I440:I441)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="443" ht="22" customHeight="1">
+      <c r="A443" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="B441" s="20" t="inlineStr">
+      <c r="B443" s="20" t="inlineStr">
         <is>
           <t>15.160.1003</t>
         </is>
       </c>
-      <c r="C441" s="8" t="inlineStr">
+      <c r="C443" s="8" t="inlineStr">
         <is>
           <t>[M26]  Ø8-Ø12 nervürlü beton çelik çubuğu — çukur, depo ve silo kaideleri</t>
         </is>
       </c>
-      <c r="D441" s="21" t="inlineStr">
-        <is>
-          <t>ton</t>
-        </is>
-      </c>
-      <c r="E441" s="22" t="n"/>
-      <c r="F441" s="22" t="n"/>
-      <c r="G441" s="22" t="n"/>
-      <c r="H441" s="22" t="n"/>
-      <c r="I441" s="22" t="n"/>
-      <c r="J441" s="22" t="n"/>
-    </row>
-    <row r="442" ht="12" customHeight="1">
-      <c r="A442" s="6" t="n"/>
-      <c r="B442" s="6" t="n"/>
-      <c r="C442" s="23" t="inlineStr">
-        <is>
-          <t>Silo kaideleri: 2.90x2.90x0.50 m³ x 2, 90 kg/m³</t>
-        </is>
-      </c>
-      <c r="D442" s="6" t="n"/>
-      <c r="E442" s="28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F442" s="29" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G442" s="29" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="H442" s="29" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I442" s="24">
-        <f>E442*F442*G442*H442*J442</f>
-        <v/>
-      </c>
-      <c r="J442" s="30" t="n">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="443">
-      <c r="A443" s="22" t="n"/>
-      <c r="B443" s="22" t="n"/>
-      <c r="C443" s="25" t="inlineStr">
-        <is>
-          <t>M26 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D443" s="26" t="inlineStr">
+      <c r="D443" s="21" t="inlineStr">
         <is>
           <t>ton</t>
         </is>
@@ -11517,208 +11520,200 @@
       <c r="G443" s="22" t="n"/>
       <c r="H443" s="22" t="n"/>
       <c r="I443" s="22" t="n"/>
-      <c r="J443" s="27">
-        <f>SUM(I442:I442)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="445" ht="20" customHeight="1">
-      <c r="A445" s="18" t="inlineStr">
+      <c r="J443" s="22" t="n"/>
+    </row>
+    <row r="444" ht="20" customHeight="1">
+      <c r="A444" s="6" t="n"/>
+      <c r="B444" s="6" t="n"/>
+      <c r="C444" s="23" t="inlineStr">
+        <is>
+          <t>Silo kaideleri — proje METRAJ tabloları: radye 198,80 + kolonlar 72,59 = 271,39 kg/kaide; 2 kaide</t>
+        </is>
+      </c>
+      <c r="D444" s="6" t="n"/>
+      <c r="E444" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F444" s="6" t="n"/>
+      <c r="G444" s="6" t="n"/>
+      <c r="H444" s="6" t="n"/>
+      <c r="I444" s="24">
+        <f>E444*J444</f>
+        <v/>
+      </c>
+      <c r="J444" s="30" t="n">
+        <v>0.27139</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="22" t="n"/>
+      <c r="B445" s="22" t="n"/>
+      <c r="C445" s="25" t="inlineStr">
+        <is>
+          <t>M26 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D445" s="26" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="E445" s="22" t="n"/>
+      <c r="F445" s="22" t="n"/>
+      <c r="G445" s="22" t="n"/>
+      <c r="H445" s="22" t="n"/>
+      <c r="I445" s="22" t="n"/>
+      <c r="J445" s="27">
+        <f>SUM(I444:I444)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="446" ht="15" customHeight="1">
+      <c r="A446" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B446" s="20" t="inlineStr">
+        <is>
+          <t>15.160.1004</t>
+        </is>
+      </c>
+      <c r="C446" s="8" t="inlineStr">
+        <is>
+          <t>[M28]  Ø14-Ø28 nervürlü beton çelik çubuğu — silo kaideleri</t>
+        </is>
+      </c>
+      <c r="D446" s="21" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="E446" s="22" t="n"/>
+      <c r="F446" s="22" t="n"/>
+      <c r="G446" s="22" t="n"/>
+      <c r="H446" s="22" t="n"/>
+      <c r="I446" s="22" t="n"/>
+      <c r="J446" s="22" t="n"/>
+    </row>
+    <row r="447" ht="20" customHeight="1">
+      <c r="A447" s="6" t="n"/>
+      <c r="B447" s="6" t="n"/>
+      <c r="C447" s="23" t="inlineStr">
+        <is>
+          <t>Proje METRAJ tabloları: radye kolon filizleri 92,70 + bodrum kat kolonları 85,70 = 178,40 kg/kaide; 2 kaide</t>
+        </is>
+      </c>
+      <c r="D447" s="6" t="n"/>
+      <c r="E447" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F447" s="6" t="n"/>
+      <c r="G447" s="6" t="n"/>
+      <c r="H447" s="6" t="n"/>
+      <c r="I447" s="24">
+        <f>E447*J447</f>
+        <v/>
+      </c>
+      <c r="J447" s="30" t="n">
+        <v>0.1784</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="22" t="n"/>
+      <c r="B448" s="22" t="n"/>
+      <c r="C448" s="25" t="inlineStr">
+        <is>
+          <t>M28 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D448" s="26" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="E448" s="22" t="n"/>
+      <c r="F448" s="22" t="n"/>
+      <c r="G448" s="22" t="n"/>
+      <c r="H448" s="22" t="n"/>
+      <c r="I448" s="22" t="n"/>
+      <c r="J448" s="27">
+        <f>SUM(I447:I447)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="450" ht="20" customHeight="1">
+      <c r="A450" s="18" t="inlineStr">
         <is>
           <t>Yapı/Bina Adı: SU DEPOSU</t>
         </is>
       </c>
     </row>
-    <row r="446" ht="28" customHeight="1">
-      <c r="A446" s="7" t="inlineStr">
+    <row r="451" ht="28" customHeight="1">
+      <c r="A451" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B446" s="7" t="inlineStr">
+      <c r="B451" s="7" t="inlineStr">
         <is>
           <t>Poz No</t>
         </is>
       </c>
-      <c r="C446" s="7" t="inlineStr">
+      <c r="C451" s="7" t="inlineStr">
         <is>
           <t>Tanımı / Ölçünün Alındığı Yer</t>
         </is>
       </c>
-      <c r="D446" s="7" t="inlineStr">
+      <c r="D451" s="7" t="inlineStr">
         <is>
           <t>Birimi</t>
         </is>
       </c>
-      <c r="E446" s="7" t="inlineStr">
+      <c r="E451" s="7" t="inlineStr">
         <is>
           <t>Adet</t>
         </is>
       </c>
-      <c r="F446" s="7" t="inlineStr">
+      <c r="F451" s="7" t="inlineStr">
         <is>
           <t>En (m)</t>
         </is>
       </c>
-      <c r="G446" s="7" t="inlineStr">
+      <c r="G451" s="7" t="inlineStr">
         <is>
           <t>Boy (m)</t>
         </is>
       </c>
-      <c r="H446" s="7" t="inlineStr">
+      <c r="H451" s="7" t="inlineStr">
         <is>
           <t>Yükseklik (m)</t>
         </is>
       </c>
-      <c r="I446" s="7" t="inlineStr">
+      <c r="I451" s="7" t="inlineStr">
         <is>
           <t>Miktar</t>
         </is>
       </c>
-      <c r="J446" s="7" t="inlineStr">
+      <c r="J451" s="7" t="inlineStr">
         <is>
           <t>Toplam Miktar</t>
         </is>
       </c>
     </row>
-    <row r="447" ht="22" customHeight="1">
-      <c r="A447" s="19" t="n">
+    <row r="452" ht="22" customHeight="1">
+      <c r="A452" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B447" s="20" t="inlineStr">
+      <c r="B452" s="20" t="inlineStr">
         <is>
           <t>15.120.1101</t>
         </is>
       </c>
-      <c r="C447" s="8" t="inlineStr">
+      <c r="C452" s="8" t="inlineStr">
         <is>
           <t>[M05]  Makine ile dar ve derin sandık kazı — ölü atma çukuru, depolar, foseptik ve silo kaideleri</t>
         </is>
       </c>
-      <c r="D447" s="21" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E447" s="22" t="n"/>
-      <c r="F447" s="22" t="n"/>
-      <c r="G447" s="22" t="n"/>
-      <c r="H447" s="22" t="n"/>
-      <c r="I447" s="22" t="n"/>
-      <c r="J447" s="22" t="n"/>
-    </row>
-    <row r="448" ht="20" customHeight="1">
-      <c r="A448" s="6" t="n"/>
-      <c r="B448" s="6" t="n"/>
-      <c r="C448" s="23" t="inlineStr">
-        <is>
-          <t>Su deposu: dış 4.00x3.00; 1,00 m çalışma payı -&gt; 6.00x5.00; derinlik 3.55 m</t>
-        </is>
-      </c>
-      <c r="D448" s="6" t="n"/>
-      <c r="E448" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F448" s="29" t="n">
-        <v>5</v>
-      </c>
-      <c r="G448" s="29" t="n">
-        <v>6</v>
-      </c>
-      <c r="H448" s="29" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="I448" s="24">
-        <f>E448*F448*G448*H448</f>
-        <v/>
-      </c>
-      <c r="J448" s="6" t="n"/>
-    </row>
-    <row r="449">
-      <c r="A449" s="22" t="n"/>
-      <c r="B449" s="22" t="n"/>
-      <c r="C449" s="25" t="inlineStr">
-        <is>
-          <t>M05 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D449" s="26" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E449" s="22" t="n"/>
-      <c r="F449" s="22" t="n"/>
-      <c r="G449" s="22" t="n"/>
-      <c r="H449" s="22" t="n"/>
-      <c r="I449" s="22" t="n"/>
-      <c r="J449" s="27">
-        <f>SUM(I448:I448)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="450" ht="22" customHeight="1">
-      <c r="A450" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="B450" s="20" t="inlineStr">
-        <is>
-          <t>15.150.1003</t>
-        </is>
-      </c>
-      <c r="C450" s="8" t="inlineStr">
-        <is>
-          <t>[M11]  C 16/20 hazır beton dökülmesi — çukur, depo, foseptik ve silo kaideleri altı grobeton</t>
-        </is>
-      </c>
-      <c r="D450" s="21" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E450" s="22" t="n"/>
-      <c r="F450" s="22" t="n"/>
-      <c r="G450" s="22" t="n"/>
-      <c r="H450" s="22" t="n"/>
-      <c r="I450" s="22" t="n"/>
-      <c r="J450" s="22" t="n"/>
-    </row>
-    <row r="451" ht="12" customHeight="1">
-      <c r="A451" s="6" t="n"/>
-      <c r="B451" s="6" t="n"/>
-      <c r="C451" s="23" t="inlineStr">
-        <is>
-          <t>Su deposu (4.00x3.00 + 0,10 taşma)</t>
-        </is>
-      </c>
-      <c r="D451" s="6" t="n"/>
-      <c r="E451" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F451" s="29" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="G451" s="29" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="H451" s="29" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I451" s="24">
-        <f>E451*F451*G451*H451</f>
-        <v/>
-      </c>
-      <c r="J451" s="6" t="n"/>
-    </row>
-    <row r="452">
-      <c r="A452" s="22" t="n"/>
-      <c r="B452" s="22" t="n"/>
-      <c r="C452" s="25" t="inlineStr">
-        <is>
-          <t>M11 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D452" s="26" t="inlineStr">
+      <c r="D452" s="21" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
@@ -11728,97 +11723,90 @@
       <c r="G452" s="22" t="n"/>
       <c r="H452" s="22" t="n"/>
       <c r="I452" s="22" t="n"/>
-      <c r="J452" s="27">
-        <f>SUM(I451:I451)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="453" ht="22" customHeight="1">
-      <c r="A453" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="B453" s="20" t="inlineStr">
-        <is>
-          <t>15.150.1005</t>
-        </is>
-      </c>
-      <c r="C453" s="8" t="inlineStr">
-        <is>
-          <t>[M16]  C 25/30 hazır beton dökülmesi — ölü atma çukuru, su ve yağmur suyu depoları</t>
-        </is>
-      </c>
-      <c r="D453" s="21" t="inlineStr">
+      <c r="J452" s="22" t="n"/>
+    </row>
+    <row r="453" ht="20" customHeight="1">
+      <c r="A453" s="6" t="n"/>
+      <c r="B453" s="6" t="n"/>
+      <c r="C453" s="23" t="inlineStr">
+        <is>
+          <t>Su deposu: dış 4.00x3.00; 1,00 m çalışma payı -&gt; 6.00x5.00; derinlik 3.55 m</t>
+        </is>
+      </c>
+      <c r="D453" s="6" t="n"/>
+      <c r="E453" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F453" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="G453" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="H453" s="29" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="I453" s="24">
+        <f>E453*F453*G453*H453</f>
+        <v/>
+      </c>
+      <c r="J453" s="6" t="n"/>
+    </row>
+    <row r="454">
+      <c r="A454" s="22" t="n"/>
+      <c r="B454" s="22" t="n"/>
+      <c r="C454" s="25" t="inlineStr">
+        <is>
+          <t>M05 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D454" s="26" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="E453" s="22" t="n"/>
-      <c r="F453" s="22" t="n"/>
-      <c r="G453" s="22" t="n"/>
-      <c r="H453" s="22" t="n"/>
-      <c r="I453" s="22" t="n"/>
-      <c r="J453" s="22" t="n"/>
-    </row>
-    <row r="454" ht="12" customHeight="1">
-      <c r="A454" s="6" t="n"/>
-      <c r="B454" s="6" t="n"/>
-      <c r="C454" s="23" t="inlineStr">
-        <is>
-          <t>Su deposu radye 30 cm (dış 4.00x3.00)</t>
-        </is>
-      </c>
-      <c r="D454" s="6" t="n"/>
-      <c r="E454" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F454" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="G454" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="H454" s="29" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I454" s="24">
-        <f>E454*F454*G454*H454</f>
-        <v/>
-      </c>
-      <c r="J454" s="6" t="n"/>
-    </row>
-    <row r="455" ht="12" customHeight="1">
-      <c r="A455" s="6" t="n"/>
-      <c r="B455" s="6" t="n"/>
-      <c r="C455" s="23" t="inlineStr">
-        <is>
-          <t>Su deposu perdeleri: orta çevre 2x(3.75+2.75) = 13.00 m</t>
-        </is>
-      </c>
-      <c r="D455" s="6" t="n"/>
-      <c r="E455" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F455" s="29" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G455" s="29" t="n">
-        <v>13</v>
-      </c>
-      <c r="H455" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="I455" s="24">
-        <f>E455*F455*G455*H455</f>
-        <v/>
-      </c>
-      <c r="J455" s="6" t="n"/>
+      <c r="E454" s="22" t="n"/>
+      <c r="F454" s="22" t="n"/>
+      <c r="G454" s="22" t="n"/>
+      <c r="H454" s="22" t="n"/>
+      <c r="I454" s="22" t="n"/>
+      <c r="J454" s="27">
+        <f>SUM(I453:I453)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="455" ht="22" customHeight="1">
+      <c r="A455" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B455" s="20" t="inlineStr">
+        <is>
+          <t>15.150.1003</t>
+        </is>
+      </c>
+      <c r="C455" s="8" t="inlineStr">
+        <is>
+          <t>[M11]  C 16/20 hazır beton dökülmesi — çukur, depo, foseptik ve silo kaideleri altı grobeton</t>
+        </is>
+      </c>
+      <c r="D455" s="21" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E455" s="22" t="n"/>
+      <c r="F455" s="22" t="n"/>
+      <c r="G455" s="22" t="n"/>
+      <c r="H455" s="22" t="n"/>
+      <c r="I455" s="22" t="n"/>
+      <c r="J455" s="22" t="n"/>
     </row>
     <row r="456" ht="12" customHeight="1">
       <c r="A456" s="6" t="n"/>
       <c r="B456" s="6" t="n"/>
       <c r="C456" s="23" t="inlineStr">
         <is>
-          <t>Su deposu üst döşemesi 15 cm</t>
+          <t>Su deposu (4.00x3.00 + 0,10 taşma)</t>
         </is>
       </c>
       <c r="D456" s="6" t="n"/>
@@ -11826,13 +11814,13 @@
         <v>1</v>
       </c>
       <c r="F456" s="29" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="G456" s="29" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="H456" s="29" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="I456" s="24">
         <f>E456*F456*G456*H456</f>
@@ -11845,7 +11833,7 @@
       <c r="B457" s="22" t="n"/>
       <c r="C457" s="25" t="inlineStr">
         <is>
-          <t>M16 TOPLAMI</t>
+          <t>M11 TOPLAMI</t>
         </is>
       </c>
       <c r="D457" s="26" t="inlineStr">
@@ -11859,27 +11847,27 @@
       <c r="H457" s="22" t="n"/>
       <c r="I457" s="22" t="n"/>
       <c r="J457" s="27">
-        <f>SUM(I454:I456)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="458" ht="15" customHeight="1">
+        <f>SUM(I456:I456)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="458" ht="22" customHeight="1">
       <c r="A458" s="19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B458" s="20" t="inlineStr">
         <is>
-          <t>15.180.1003</t>
+          <t>15.150.1005</t>
         </is>
       </c>
       <c r="C458" s="8" t="inlineStr">
         <is>
-          <t>[M20]  Plywood ile düz yüzeyli betonarme kalıbı — çukur ve depolar</t>
+          <t>[M16]  C 25/30 hazır beton dökülmesi — ölü atma çukuru, su ve yağmur suyu depoları</t>
         </is>
       </c>
       <c r="D458" s="21" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E458" s="22" t="n"/>
@@ -11894,22 +11882,24 @@
       <c r="B459" s="6" t="n"/>
       <c r="C459" s="23" t="inlineStr">
         <is>
-          <t>Su deposu radye çevresi 2x(4.00+3.00) = 14.00 m x 0,40</t>
+          <t>Su deposu radye 30 cm (dış 4.00x3.00)</t>
         </is>
       </c>
       <c r="D459" s="6" t="n"/>
       <c r="E459" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F459" s="6" t="n"/>
+      <c r="F459" s="29" t="n">
+        <v>3</v>
+      </c>
       <c r="G459" s="29" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H459" s="29" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="I459" s="24">
-        <f>E459*G459*H459</f>
+        <f>E459*F459*G459*H459</f>
         <v/>
       </c>
       <c r="J459" s="6" t="n"/>
@@ -11919,14 +11909,16 @@
       <c r="B460" s="6" t="n"/>
       <c r="C460" s="23" t="inlineStr">
         <is>
-          <t>Su deposu perde iki yüz (13.00 m x 3.00 m)</t>
+          <t>Su deposu perdeleri: orta çevre 2x(3.75+2.75) = 13.00 m</t>
         </is>
       </c>
       <c r="D460" s="6" t="n"/>
       <c r="E460" s="28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F460" s="6" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="F460" s="29" t="n">
+        <v>0.25</v>
+      </c>
       <c r="G460" s="29" t="n">
         <v>13</v>
       </c>
@@ -11934,7 +11926,7 @@
         <v>3</v>
       </c>
       <c r="I460" s="24">
-        <f>E460*G460*H460</f>
+        <f>E460*F460*G460*H460</f>
         <v/>
       </c>
       <c r="J460" s="6" t="n"/>
@@ -11944,7 +11936,7 @@
       <c r="B461" s="6" t="n"/>
       <c r="C461" s="23" t="inlineStr">
         <is>
-          <t>Su deposu tavan kalıbı</t>
+          <t>Su deposu üst döşemesi 15 cm</t>
         </is>
       </c>
       <c r="D461" s="6" t="n"/>
@@ -11957,9 +11949,11 @@
       <c r="G461" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="H461" s="6" t="n"/>
+      <c r="H461" s="29" t="n">
+        <v>0.15</v>
+      </c>
       <c r="I461" s="24">
-        <f>E461*F461*G461</f>
+        <f>E461*F461*G461*H461</f>
         <v/>
       </c>
       <c r="J461" s="6" t="n"/>
@@ -11969,12 +11963,12 @@
       <c r="B462" s="22" t="n"/>
       <c r="C462" s="25" t="inlineStr">
         <is>
-          <t>M20 TOPLAMI</t>
+          <t>M16 TOPLAMI</t>
         </is>
       </c>
       <c r="D462" s="26" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E462" s="22" t="n"/>
@@ -11987,23 +11981,23 @@
         <v/>
       </c>
     </row>
-    <row r="463" ht="22" customHeight="1">
+    <row r="463" ht="15" customHeight="1">
       <c r="A463" s="19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B463" s="20" t="inlineStr">
         <is>
-          <t>15.160.1003</t>
+          <t>15.180.1003</t>
         </is>
       </c>
       <c r="C463" s="8" t="inlineStr">
         <is>
-          <t>[M26]  Ø8-Ø12 nervürlü beton çelik çubuğu — çukur, depo ve silo kaideleri</t>
+          <t>[M20]  Plywood ile düz yüzeyli betonarme kalıbı — çukur ve depolar</t>
         </is>
       </c>
       <c r="D463" s="21" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E463" s="22" t="n"/>
@@ -12013,12 +12007,12 @@
       <c r="I463" s="22" t="n"/>
       <c r="J463" s="22" t="n"/>
     </row>
-    <row r="464" ht="20" customHeight="1">
+    <row r="464" ht="12" customHeight="1">
       <c r="A464" s="6" t="n"/>
       <c r="B464" s="6" t="n"/>
       <c r="C464" s="23" t="inlineStr">
         <is>
-          <t>Su deposu radye ve döşeme — proje metrajı 223,70+32,90 = 256,60 kg</t>
+          <t>Su deposu radye çevresi 2x(4.00+3.00) = 14.00 m x 0,40</t>
         </is>
       </c>
       <c r="D464" s="6" t="n"/>
@@ -12026,31 +12020,31 @@
         <v>1</v>
       </c>
       <c r="F464" s="6" t="n"/>
-      <c r="G464" s="6" t="n"/>
-      <c r="H464" s="6" t="n"/>
+      <c r="G464" s="29" t="n">
+        <v>14</v>
+      </c>
+      <c r="H464" s="29" t="n">
+        <v>0.4</v>
+      </c>
       <c r="I464" s="24">
-        <f>E464*J464</f>
-        <v/>
-      </c>
-      <c r="J464" s="30" t="n">
-        <v>0.2566</v>
-      </c>
+        <f>E464*G464*H464</f>
+        <v/>
+      </c>
+      <c r="J464" s="6" t="n"/>
     </row>
     <row r="465" ht="12" customHeight="1">
       <c r="A465" s="6" t="n"/>
       <c r="B465" s="6" t="n"/>
       <c r="C465" s="23" t="inlineStr">
         <is>
-          <t>Su deposu perdeleri: 13.00x0,25x3.00 m³, 100 kg/m³</t>
+          <t>Su deposu perde iki yüz (13.00 m x 3.00 m)</t>
         </is>
       </c>
       <c r="D465" s="6" t="n"/>
       <c r="E465" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F465" s="29" t="n">
-        <v>0.25</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F465" s="6" t="n"/>
       <c r="G465" s="29" t="n">
         <v>13</v>
       </c>
@@ -12058,233 +12052,234 @@
         <v>3</v>
       </c>
       <c r="I465" s="24">
-        <f>E465*F465*G465*H465*J465</f>
-        <v/>
-      </c>
-      <c r="J465" s="30" t="n">
+        <f>E465*G465*H465</f>
+        <v/>
+      </c>
+      <c r="J465" s="6" t="n"/>
+    </row>
+    <row r="466" ht="12" customHeight="1">
+      <c r="A466" s="6" t="n"/>
+      <c r="B466" s="6" t="n"/>
+      <c r="C466" s="23" t="inlineStr">
+        <is>
+          <t>Su deposu tavan kalıbı</t>
+        </is>
+      </c>
+      <c r="D466" s="6" t="n"/>
+      <c r="E466" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F466" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G466" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="H466" s="6" t="n"/>
+      <c r="I466" s="24">
+        <f>E466*F466*G466</f>
+        <v/>
+      </c>
+      <c r="J466" s="6" t="n"/>
+    </row>
+    <row r="467">
+      <c r="A467" s="22" t="n"/>
+      <c r="B467" s="22" t="n"/>
+      <c r="C467" s="25" t="inlineStr">
+        <is>
+          <t>M20 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D467" s="26" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E467" s="22" t="n"/>
+      <c r="F467" s="22" t="n"/>
+      <c r="G467" s="22" t="n"/>
+      <c r="H467" s="22" t="n"/>
+      <c r="I467" s="22" t="n"/>
+      <c r="J467" s="27">
+        <f>SUM(I464:I466)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="468" ht="22" customHeight="1">
+      <c r="A468" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="B468" s="20" t="inlineStr">
+        <is>
+          <t>15.160.1003</t>
+        </is>
+      </c>
+      <c r="C468" s="8" t="inlineStr">
+        <is>
+          <t>[M26]  Ø8-Ø12 nervürlü beton çelik çubuğu — çukur, depo ve silo kaideleri</t>
+        </is>
+      </c>
+      <c r="D468" s="21" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="E468" s="22" t="n"/>
+      <c r="F468" s="22" t="n"/>
+      <c r="G468" s="22" t="n"/>
+      <c r="H468" s="22" t="n"/>
+      <c r="I468" s="22" t="n"/>
+      <c r="J468" s="22" t="n"/>
+    </row>
+    <row r="469" ht="20" customHeight="1">
+      <c r="A469" s="6" t="n"/>
+      <c r="B469" s="6" t="n"/>
+      <c r="C469" s="23" t="inlineStr">
+        <is>
+          <t>Su deposu radye ve döşeme — proje metrajı 223,70+32,90 = 256,60 kg</t>
+        </is>
+      </c>
+      <c r="D469" s="6" t="n"/>
+      <c r="E469" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F469" s="6" t="n"/>
+      <c r="G469" s="6" t="n"/>
+      <c r="H469" s="6" t="n"/>
+      <c r="I469" s="24">
+        <f>E469*J469</f>
+        <v/>
+      </c>
+      <c r="J469" s="30" t="n">
+        <v>0.2566</v>
+      </c>
+    </row>
+    <row r="470" ht="12" customHeight="1">
+      <c r="A470" s="6" t="n"/>
+      <c r="B470" s="6" t="n"/>
+      <c r="C470" s="23" t="inlineStr">
+        <is>
+          <t>Su deposu perdeleri: 13.00x0,25x3.00 m³, 100 kg/m³</t>
+        </is>
+      </c>
+      <c r="D470" s="6" t="n"/>
+      <c r="E470" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F470" s="29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G470" s="29" t="n">
+        <v>13</v>
+      </c>
+      <c r="H470" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="I470" s="24">
+        <f>E470*F470*G470*H470*J470</f>
+        <v/>
+      </c>
+      <c r="J470" s="30" t="n">
         <v>0.1</v>
       </c>
     </row>
-    <row r="466">
-      <c r="A466" s="22" t="n"/>
-      <c r="B466" s="22" t="n"/>
-      <c r="C466" s="25" t="inlineStr">
+    <row r="471">
+      <c r="A471" s="22" t="n"/>
+      <c r="B471" s="22" t="n"/>
+      <c r="C471" s="25" t="inlineStr">
         <is>
           <t>M26 TOPLAMI</t>
         </is>
       </c>
-      <c r="D466" s="26" t="inlineStr">
+      <c r="D471" s="26" t="inlineStr">
         <is>
           <t>ton</t>
         </is>
       </c>
-      <c r="E466" s="22" t="n"/>
-      <c r="F466" s="22" t="n"/>
-      <c r="G466" s="22" t="n"/>
-      <c r="H466" s="22" t="n"/>
-      <c r="I466" s="22" t="n"/>
-      <c r="J466" s="27">
-        <f>SUM(I464:I465)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="468" ht="20" customHeight="1">
-      <c r="A468" s="18" t="inlineStr">
+      <c r="E471" s="22" t="n"/>
+      <c r="F471" s="22" t="n"/>
+      <c r="G471" s="22" t="n"/>
+      <c r="H471" s="22" t="n"/>
+      <c r="I471" s="22" t="n"/>
+      <c r="J471" s="27">
+        <f>SUM(I469:I470)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="473" ht="20" customHeight="1">
+      <c r="A473" s="18" t="inlineStr">
         <is>
           <t>Yapı/Bina Adı: YAĞMUR SUYU DEPOSU</t>
         </is>
       </c>
     </row>
-    <row r="469" ht="28" customHeight="1">
-      <c r="A469" s="7" t="inlineStr">
+    <row r="474" ht="28" customHeight="1">
+      <c r="A474" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B469" s="7" t="inlineStr">
+      <c r="B474" s="7" t="inlineStr">
         <is>
           <t>Poz No</t>
         </is>
       </c>
-      <c r="C469" s="7" t="inlineStr">
+      <c r="C474" s="7" t="inlineStr">
         <is>
           <t>Tanımı / Ölçünün Alındığı Yer</t>
         </is>
       </c>
-      <c r="D469" s="7" t="inlineStr">
+      <c r="D474" s="7" t="inlineStr">
         <is>
           <t>Birimi</t>
         </is>
       </c>
-      <c r="E469" s="7" t="inlineStr">
+      <c r="E474" s="7" t="inlineStr">
         <is>
           <t>Adet</t>
         </is>
       </c>
-      <c r="F469" s="7" t="inlineStr">
+      <c r="F474" s="7" t="inlineStr">
         <is>
           <t>En (m)</t>
         </is>
       </c>
-      <c r="G469" s="7" t="inlineStr">
+      <c r="G474" s="7" t="inlineStr">
         <is>
           <t>Boy (m)</t>
         </is>
       </c>
-      <c r="H469" s="7" t="inlineStr">
+      <c r="H474" s="7" t="inlineStr">
         <is>
           <t>Yükseklik (m)</t>
         </is>
       </c>
-      <c r="I469" s="7" t="inlineStr">
+      <c r="I474" s="7" t="inlineStr">
         <is>
           <t>Miktar</t>
         </is>
       </c>
-      <c r="J469" s="7" t="inlineStr">
+      <c r="J474" s="7" t="inlineStr">
         <is>
           <t>Toplam Miktar</t>
         </is>
       </c>
     </row>
-    <row r="470" ht="22" customHeight="1">
-      <c r="A470" s="19" t="n">
+    <row r="475" ht="22" customHeight="1">
+      <c r="A475" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B470" s="20" t="inlineStr">
+      <c r="B475" s="20" t="inlineStr">
         <is>
           <t>15.120.1101</t>
         </is>
       </c>
-      <c r="C470" s="8" t="inlineStr">
+      <c r="C475" s="8" t="inlineStr">
         <is>
           <t>[M05]  Makine ile dar ve derin sandık kazı — ölü atma çukuru, depolar, foseptik ve silo kaideleri</t>
         </is>
       </c>
-      <c r="D470" s="21" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E470" s="22" t="n"/>
-      <c r="F470" s="22" t="n"/>
-      <c r="G470" s="22" t="n"/>
-      <c r="H470" s="22" t="n"/>
-      <c r="I470" s="22" t="n"/>
-      <c r="J470" s="22" t="n"/>
-    </row>
-    <row r="471" ht="20" customHeight="1">
-      <c r="A471" s="6" t="n"/>
-      <c r="B471" s="6" t="n"/>
-      <c r="C471" s="23" t="inlineStr">
-        <is>
-          <t>Yağmur suyu deposu: dış 3.00x3.00; 1,00 m çalışma payı -&gt; 5.00x5.00; derinlik 3.55 m</t>
-        </is>
-      </c>
-      <c r="D471" s="6" t="n"/>
-      <c r="E471" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F471" s="29" t="n">
-        <v>5</v>
-      </c>
-      <c r="G471" s="29" t="n">
-        <v>5</v>
-      </c>
-      <c r="H471" s="29" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="I471" s="24">
-        <f>E471*F471*G471*H471</f>
-        <v/>
-      </c>
-      <c r="J471" s="6" t="n"/>
-    </row>
-    <row r="472">
-      <c r="A472" s="22" t="n"/>
-      <c r="B472" s="22" t="n"/>
-      <c r="C472" s="25" t="inlineStr">
-        <is>
-          <t>M05 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D472" s="26" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E472" s="22" t="n"/>
-      <c r="F472" s="22" t="n"/>
-      <c r="G472" s="22" t="n"/>
-      <c r="H472" s="22" t="n"/>
-      <c r="I472" s="22" t="n"/>
-      <c r="J472" s="27">
-        <f>SUM(I471:I471)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="473" ht="22" customHeight="1">
-      <c r="A473" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="B473" s="20" t="inlineStr">
-        <is>
-          <t>15.150.1003</t>
-        </is>
-      </c>
-      <c r="C473" s="8" t="inlineStr">
-        <is>
-          <t>[M11]  C 16/20 hazır beton dökülmesi — çukur, depo, foseptik ve silo kaideleri altı grobeton</t>
-        </is>
-      </c>
-      <c r="D473" s="21" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E473" s="22" t="n"/>
-      <c r="F473" s="22" t="n"/>
-      <c r="G473" s="22" t="n"/>
-      <c r="H473" s="22" t="n"/>
-      <c r="I473" s="22" t="n"/>
-      <c r="J473" s="22" t="n"/>
-    </row>
-    <row r="474" ht="12" customHeight="1">
-      <c r="A474" s="6" t="n"/>
-      <c r="B474" s="6" t="n"/>
-      <c r="C474" s="23" t="inlineStr">
-        <is>
-          <t>Yağmur suyu deposu (3.00x3.00 + 0,10 taşma)</t>
-        </is>
-      </c>
-      <c r="D474" s="6" t="n"/>
-      <c r="E474" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F474" s="29" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="G474" s="29" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="H474" s="29" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I474" s="24">
-        <f>E474*F474*G474*H474</f>
-        <v/>
-      </c>
-      <c r="J474" s="6" t="n"/>
-    </row>
-    <row r="475">
-      <c r="A475" s="22" t="n"/>
-      <c r="B475" s="22" t="n"/>
-      <c r="C475" s="25" t="inlineStr">
-        <is>
-          <t>M11 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D475" s="26" t="inlineStr">
+      <c r="D475" s="21" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
@@ -12294,97 +12289,90 @@
       <c r="G475" s="22" t="n"/>
       <c r="H475" s="22" t="n"/>
       <c r="I475" s="22" t="n"/>
-      <c r="J475" s="27">
-        <f>SUM(I474:I474)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="476" ht="22" customHeight="1">
-      <c r="A476" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="B476" s="20" t="inlineStr">
-        <is>
-          <t>15.150.1005</t>
-        </is>
-      </c>
-      <c r="C476" s="8" t="inlineStr">
-        <is>
-          <t>[M16]  C 25/30 hazır beton dökülmesi — ölü atma çukuru, su ve yağmur suyu depoları</t>
-        </is>
-      </c>
-      <c r="D476" s="21" t="inlineStr">
+      <c r="J475" s="22" t="n"/>
+    </row>
+    <row r="476" ht="20" customHeight="1">
+      <c r="A476" s="6" t="n"/>
+      <c r="B476" s="6" t="n"/>
+      <c r="C476" s="23" t="inlineStr">
+        <is>
+          <t>Yağmur suyu deposu: dış 3.00x3.00; 1,00 m çalışma payı -&gt; 5.00x5.00; derinlik 3.55 m</t>
+        </is>
+      </c>
+      <c r="D476" s="6" t="n"/>
+      <c r="E476" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F476" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="G476" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="H476" s="29" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="I476" s="24">
+        <f>E476*F476*G476*H476</f>
+        <v/>
+      </c>
+      <c r="J476" s="6" t="n"/>
+    </row>
+    <row r="477">
+      <c r="A477" s="22" t="n"/>
+      <c r="B477" s="22" t="n"/>
+      <c r="C477" s="25" t="inlineStr">
+        <is>
+          <t>M05 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D477" s="26" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="E476" s="22" t="n"/>
-      <c r="F476" s="22" t="n"/>
-      <c r="G476" s="22" t="n"/>
-      <c r="H476" s="22" t="n"/>
-      <c r="I476" s="22" t="n"/>
-      <c r="J476" s="22" t="n"/>
-    </row>
-    <row r="477" ht="12" customHeight="1">
-      <c r="A477" s="6" t="n"/>
-      <c r="B477" s="6" t="n"/>
-      <c r="C477" s="23" t="inlineStr">
-        <is>
-          <t>Yağmur suyu deposu radye 30 cm (dış 3.00x3.00)</t>
-        </is>
-      </c>
-      <c r="D477" s="6" t="n"/>
-      <c r="E477" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F477" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="G477" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="H477" s="29" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I477" s="24">
-        <f>E477*F477*G477*H477</f>
-        <v/>
-      </c>
-      <c r="J477" s="6" t="n"/>
-    </row>
-    <row r="478" ht="20" customHeight="1">
-      <c r="A478" s="6" t="n"/>
-      <c r="B478" s="6" t="n"/>
-      <c r="C478" s="23" t="inlineStr">
-        <is>
-          <t>Yağmur suyu deposu perdeleri: orta çevre 2x(2.75+2.75) = 11.00 m</t>
-        </is>
-      </c>
-      <c r="D478" s="6" t="n"/>
-      <c r="E478" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F478" s="29" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G478" s="29" t="n">
-        <v>11</v>
-      </c>
-      <c r="H478" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="I478" s="24">
-        <f>E478*F478*G478*H478</f>
-        <v/>
-      </c>
-      <c r="J478" s="6" t="n"/>
+      <c r="E477" s="22" t="n"/>
+      <c r="F477" s="22" t="n"/>
+      <c r="G477" s="22" t="n"/>
+      <c r="H477" s="22" t="n"/>
+      <c r="I477" s="22" t="n"/>
+      <c r="J477" s="27">
+        <f>SUM(I476:I476)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="478" ht="22" customHeight="1">
+      <c r="A478" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B478" s="20" t="inlineStr">
+        <is>
+          <t>15.150.1003</t>
+        </is>
+      </c>
+      <c r="C478" s="8" t="inlineStr">
+        <is>
+          <t>[M11]  C 16/20 hazır beton dökülmesi — çukur, depo, foseptik ve silo kaideleri altı grobeton</t>
+        </is>
+      </c>
+      <c r="D478" s="21" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E478" s="22" t="n"/>
+      <c r="F478" s="22" t="n"/>
+      <c r="G478" s="22" t="n"/>
+      <c r="H478" s="22" t="n"/>
+      <c r="I478" s="22" t="n"/>
+      <c r="J478" s="22" t="n"/>
     </row>
     <row r="479" ht="12" customHeight="1">
       <c r="A479" s="6" t="n"/>
       <c r="B479" s="6" t="n"/>
       <c r="C479" s="23" t="inlineStr">
         <is>
-          <t>Yağmur suyu deposu üst döşemesi 15 cm</t>
+          <t>Yağmur suyu deposu (3.00x3.00 + 0,10 taşma)</t>
         </is>
       </c>
       <c r="D479" s="6" t="n"/>
@@ -12392,13 +12380,13 @@
         <v>1</v>
       </c>
       <c r="F479" s="29" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="G479" s="29" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H479" s="29" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="I479" s="24">
         <f>E479*F479*G479*H479</f>
@@ -12411,7 +12399,7 @@
       <c r="B480" s="22" t="n"/>
       <c r="C480" s="25" t="inlineStr">
         <is>
-          <t>M16 TOPLAMI</t>
+          <t>M11 TOPLAMI</t>
         </is>
       </c>
       <c r="D480" s="26" t="inlineStr">
@@ -12425,27 +12413,27 @@
       <c r="H480" s="22" t="n"/>
       <c r="I480" s="22" t="n"/>
       <c r="J480" s="27">
-        <f>SUM(I477:I479)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="481" ht="15" customHeight="1">
+        <f>SUM(I479:I479)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="481" ht="22" customHeight="1">
       <c r="A481" s="19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B481" s="20" t="inlineStr">
         <is>
-          <t>15.180.1003</t>
+          <t>15.150.1005</t>
         </is>
       </c>
       <c r="C481" s="8" t="inlineStr">
         <is>
-          <t>[M20]  Plywood ile düz yüzeyli betonarme kalıbı — çukur ve depolar</t>
+          <t>[M16]  C 25/30 hazır beton dökülmesi — ölü atma çukuru, su ve yağmur suyu depoları</t>
         </is>
       </c>
       <c r="D481" s="21" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E481" s="22" t="n"/>
@@ -12455,44 +12443,48 @@
       <c r="I481" s="22" t="n"/>
       <c r="J481" s="22" t="n"/>
     </row>
-    <row r="482" ht="20" customHeight="1">
+    <row r="482" ht="12" customHeight="1">
       <c r="A482" s="6" t="n"/>
       <c r="B482" s="6" t="n"/>
       <c r="C482" s="23" t="inlineStr">
         <is>
-          <t>Yağmur suyu deposu radye çevresi 2x(3.00+3.00) = 12.00 m x 0,40</t>
+          <t>Yağmur suyu deposu radye 30 cm (dış 3.00x3.00)</t>
         </is>
       </c>
       <c r="D482" s="6" t="n"/>
       <c r="E482" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F482" s="6" t="n"/>
+      <c r="F482" s="29" t="n">
+        <v>3</v>
+      </c>
       <c r="G482" s="29" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H482" s="29" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="I482" s="24">
-        <f>E482*G482*H482</f>
+        <f>E482*F482*G482*H482</f>
         <v/>
       </c>
       <c r="J482" s="6" t="n"/>
     </row>
-    <row r="483" ht="12" customHeight="1">
+    <row r="483" ht="20" customHeight="1">
       <c r="A483" s="6" t="n"/>
       <c r="B483" s="6" t="n"/>
       <c r="C483" s="23" t="inlineStr">
         <is>
-          <t>Yağmur suyu deposu perde iki yüz (11.00 m x 3.00 m)</t>
+          <t>Yağmur suyu deposu perdeleri: orta çevre 2x(2.75+2.75) = 11.00 m</t>
         </is>
       </c>
       <c r="D483" s="6" t="n"/>
       <c r="E483" s="28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F483" s="6" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="F483" s="29" t="n">
+        <v>0.25</v>
+      </c>
       <c r="G483" s="29" t="n">
         <v>11</v>
       </c>
@@ -12500,7 +12492,7 @@
         <v>3</v>
       </c>
       <c r="I483" s="24">
-        <f>E483*G483*H483</f>
+        <f>E483*F483*G483*H483</f>
         <v/>
       </c>
       <c r="J483" s="6" t="n"/>
@@ -12510,7 +12502,7 @@
       <c r="B484" s="6" t="n"/>
       <c r="C484" s="23" t="inlineStr">
         <is>
-          <t>Yağmur suyu deposu tavan kalıbı</t>
+          <t>Yağmur suyu deposu üst döşemesi 15 cm</t>
         </is>
       </c>
       <c r="D484" s="6" t="n"/>
@@ -12523,9 +12515,11 @@
       <c r="G484" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="H484" s="6" t="n"/>
+      <c r="H484" s="29" t="n">
+        <v>0.15</v>
+      </c>
       <c r="I484" s="24">
-        <f>E484*F484*G484</f>
+        <f>E484*F484*G484*H484</f>
         <v/>
       </c>
       <c r="J484" s="6" t="n"/>
@@ -12535,12 +12529,12 @@
       <c r="B485" s="22" t="n"/>
       <c r="C485" s="25" t="inlineStr">
         <is>
-          <t>M20 TOPLAMI</t>
+          <t>M16 TOPLAMI</t>
         </is>
       </c>
       <c r="D485" s="26" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E485" s="22" t="n"/>
@@ -12553,23 +12547,23 @@
         <v/>
       </c>
     </row>
-    <row r="486" ht="22" customHeight="1">
+    <row r="486" ht="15" customHeight="1">
       <c r="A486" s="19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B486" s="20" t="inlineStr">
         <is>
-          <t>15.160.1003</t>
+          <t>15.180.1003</t>
         </is>
       </c>
       <c r="C486" s="8" t="inlineStr">
         <is>
-          <t>[M26]  Ø8-Ø12 nervürlü beton çelik çubuğu — çukur, depo ve silo kaideleri</t>
+          <t>[M20]  Plywood ile düz yüzeyli betonarme kalıbı — çukur ve depolar</t>
         </is>
       </c>
       <c r="D486" s="21" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E486" s="22" t="n"/>
@@ -12579,50 +12573,44 @@
       <c r="I486" s="22" t="n"/>
       <c r="J486" s="22" t="n"/>
     </row>
-    <row r="487" ht="12" customHeight="1">
+    <row r="487" ht="20" customHeight="1">
       <c r="A487" s="6" t="n"/>
       <c r="B487" s="6" t="n"/>
       <c r="C487" s="23" t="inlineStr">
         <is>
-          <t>Yağmur suyu deposu radyesi: 3.00x3.00x0,30 m³, 100 kg/m³</t>
+          <t>Yağmur suyu deposu radye çevresi 2x(3.00+3.00) = 12.00 m x 0,40</t>
         </is>
       </c>
       <c r="D487" s="6" t="n"/>
       <c r="E487" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F487" s="29" t="n">
-        <v>3</v>
-      </c>
+      <c r="F487" s="6" t="n"/>
       <c r="G487" s="29" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H487" s="29" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I487" s="24">
-        <f>E487*F487*G487*H487*J487</f>
-        <v/>
-      </c>
-      <c r="J487" s="30" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="488" ht="20" customHeight="1">
+        <f>E487*G487*H487</f>
+        <v/>
+      </c>
+      <c r="J487" s="6" t="n"/>
+    </row>
+    <row r="488" ht="12" customHeight="1">
       <c r="A488" s="6" t="n"/>
       <c r="B488" s="6" t="n"/>
       <c r="C488" s="23" t="inlineStr">
         <is>
-          <t>Yağmur suyu deposu perdeleri: 11.00x0,25x3.00 m³, 100 kg/m³</t>
+          <t>Yağmur suyu deposu perde iki yüz (11.00 m x 3.00 m)</t>
         </is>
       </c>
       <c r="D488" s="6" t="n"/>
       <c r="E488" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F488" s="29" t="n">
-        <v>0.25</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F488" s="6" t="n"/>
       <c r="G488" s="29" t="n">
         <v>11</v>
       </c>
@@ -12630,19 +12618,17 @@
         <v>3</v>
       </c>
       <c r="I488" s="24">
-        <f>E488*F488*G488*H488*J488</f>
-        <v/>
-      </c>
-      <c r="J488" s="30" t="n">
-        <v>0.1</v>
-      </c>
+        <f>E488*G488*H488</f>
+        <v/>
+      </c>
+      <c r="J488" s="6" t="n"/>
     </row>
     <row r="489" ht="12" customHeight="1">
       <c r="A489" s="6" t="n"/>
       <c r="B489" s="6" t="n"/>
       <c r="C489" s="23" t="inlineStr">
         <is>
-          <t>Yağmur suyu deposu döşemesi: 3.00x3.00x0,15 m³, 100 kg/m³</t>
+          <t>Yağmur suyu deposu tavan kalıbı</t>
         </is>
       </c>
       <c r="D489" s="6" t="n"/>
@@ -12655,28 +12641,24 @@
       <c r="G489" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="H489" s="29" t="n">
-        <v>0.15</v>
-      </c>
+      <c r="H489" s="6" t="n"/>
       <c r="I489" s="24">
-        <f>E489*F489*G489*H489*J489</f>
-        <v/>
-      </c>
-      <c r="J489" s="30" t="n">
-        <v>0.1</v>
-      </c>
+        <f>E489*F489*G489</f>
+        <v/>
+      </c>
+      <c r="J489" s="6" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="22" t="n"/>
       <c r="B490" s="22" t="n"/>
       <c r="C490" s="25" t="inlineStr">
         <is>
-          <t>M26 TOPLAMI</t>
+          <t>M20 TOPLAMI</t>
         </is>
       </c>
       <c r="D490" s="26" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E490" s="22" t="n"/>
@@ -12689,253 +12671,265 @@
         <v/>
       </c>
     </row>
-    <row r="492" ht="20" customHeight="1">
-      <c r="A492" s="18" t="inlineStr">
+    <row r="491" ht="22" customHeight="1">
+      <c r="A491" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="B491" s="20" t="inlineStr">
+        <is>
+          <t>15.160.1003</t>
+        </is>
+      </c>
+      <c r="C491" s="8" t="inlineStr">
+        <is>
+          <t>[M26]  Ø8-Ø12 nervürlü beton çelik çubuğu — çukur, depo ve silo kaideleri</t>
+        </is>
+      </c>
+      <c r="D491" s="21" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="E491" s="22" t="n"/>
+      <c r="F491" s="22" t="n"/>
+      <c r="G491" s="22" t="n"/>
+      <c r="H491" s="22" t="n"/>
+      <c r="I491" s="22" t="n"/>
+      <c r="J491" s="22" t="n"/>
+    </row>
+    <row r="492" ht="12" customHeight="1">
+      <c r="A492" s="6" t="n"/>
+      <c r="B492" s="6" t="n"/>
+      <c r="C492" s="23" t="inlineStr">
+        <is>
+          <t>Yağmur suyu deposu radyesi: 3.00x3.00x0,30 m³, 100 kg/m³</t>
+        </is>
+      </c>
+      <c r="D492" s="6" t="n"/>
+      <c r="E492" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F492" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G492" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="H492" s="29" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I492" s="24">
+        <f>E492*F492*G492*H492*J492</f>
+        <v/>
+      </c>
+      <c r="J492" s="30" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="493" ht="20" customHeight="1">
+      <c r="A493" s="6" t="n"/>
+      <c r="B493" s="6" t="n"/>
+      <c r="C493" s="23" t="inlineStr">
+        <is>
+          <t>Yağmur suyu deposu perdeleri: 11.00x0,25x3.00 m³, 100 kg/m³</t>
+        </is>
+      </c>
+      <c r="D493" s="6" t="n"/>
+      <c r="E493" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F493" s="29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G493" s="29" t="n">
+        <v>11</v>
+      </c>
+      <c r="H493" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="I493" s="24">
+        <f>E493*F493*G493*H493*J493</f>
+        <v/>
+      </c>
+      <c r="J493" s="30" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="494" ht="12" customHeight="1">
+      <c r="A494" s="6" t="n"/>
+      <c r="B494" s="6" t="n"/>
+      <c r="C494" s="23" t="inlineStr">
+        <is>
+          <t>Yağmur suyu deposu döşemesi: 3.00x3.00x0,15 m³, 100 kg/m³</t>
+        </is>
+      </c>
+      <c r="D494" s="6" t="n"/>
+      <c r="E494" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F494" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G494" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="H494" s="29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I494" s="24">
+        <f>E494*F494*G494*H494*J494</f>
+        <v/>
+      </c>
+      <c r="J494" s="30" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="22" t="n"/>
+      <c r="B495" s="22" t="n"/>
+      <c r="C495" s="25" t="inlineStr">
+        <is>
+          <t>M26 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D495" s="26" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="E495" s="22" t="n"/>
+      <c r="F495" s="22" t="n"/>
+      <c r="G495" s="22" t="n"/>
+      <c r="H495" s="22" t="n"/>
+      <c r="I495" s="22" t="n"/>
+      <c r="J495" s="27">
+        <f>SUM(I492:I494)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="497" ht="20" customHeight="1">
+      <c r="A497" s="18" t="inlineStr">
         <is>
           <t>Yapı/Bina Adı: ÇEVRE DÜZENLEMESI VE SAHA ALTYAPISI</t>
         </is>
       </c>
     </row>
-    <row r="493" ht="28" customHeight="1">
-      <c r="A493" s="7" t="inlineStr">
+    <row r="498" ht="28" customHeight="1">
+      <c r="A498" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B493" s="7" t="inlineStr">
+      <c r="B498" s="7" t="inlineStr">
         <is>
           <t>Poz No</t>
         </is>
       </c>
-      <c r="C493" s="7" t="inlineStr">
+      <c r="C498" s="7" t="inlineStr">
         <is>
           <t>Tanımı / Ölçünün Alındığı Yer</t>
         </is>
       </c>
-      <c r="D493" s="7" t="inlineStr">
+      <c r="D498" s="7" t="inlineStr">
         <is>
           <t>Birimi</t>
         </is>
       </c>
-      <c r="E493" s="7" t="inlineStr">
+      <c r="E498" s="7" t="inlineStr">
         <is>
           <t>Adet</t>
         </is>
       </c>
-      <c r="F493" s="7" t="inlineStr">
+      <c r="F498" s="7" t="inlineStr">
         <is>
           <t>En (m)</t>
         </is>
       </c>
-      <c r="G493" s="7" t="inlineStr">
+      <c r="G498" s="7" t="inlineStr">
         <is>
           <t>Boy (m)</t>
         </is>
       </c>
-      <c r="H493" s="7" t="inlineStr">
+      <c r="H498" s="7" t="inlineStr">
         <is>
           <t>Yükseklik (m)</t>
         </is>
       </c>
-      <c r="I493" s="7" t="inlineStr">
+      <c r="I498" s="7" t="inlineStr">
         <is>
           <t>Miktar</t>
         </is>
       </c>
-      <c r="J493" s="7" t="inlineStr">
+      <c r="J498" s="7" t="inlineStr">
         <is>
           <t>Toplam Miktar</t>
         </is>
       </c>
     </row>
-    <row r="494" ht="15" customHeight="1">
-      <c r="A494" s="19" t="n">
+    <row r="499" ht="15" customHeight="1">
+      <c r="A499" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B494" s="20" t="inlineStr">
+      <c r="B499" s="20" t="inlineStr">
         <is>
           <t>15.120.1001</t>
         </is>
       </c>
-      <c r="C494" s="8" t="inlineStr">
+      <c r="C499" s="8" t="inlineStr">
         <is>
           <t>[M02]  Makine ile kaba tesviye kazısı — tesis içi yol güzergâhı</t>
         </is>
       </c>
-      <c r="D494" s="21" t="inlineStr">
+      <c r="D499" s="21" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="E494" s="22" t="n"/>
-      <c r="F494" s="22" t="n"/>
-      <c r="G494" s="22" t="n"/>
-      <c r="H494" s="22" t="n"/>
-      <c r="I494" s="22" t="n"/>
-      <c r="J494" s="22" t="n"/>
-    </row>
-    <row r="495" ht="20" customHeight="1">
-      <c r="A495" s="6" t="n"/>
-      <c r="B495" s="6" t="n"/>
-      <c r="C495" s="23" t="inlineStr">
+      <c r="E499" s="22" t="n"/>
+      <c r="F499" s="22" t="n"/>
+      <c r="G499" s="22" t="n"/>
+      <c r="H499" s="22" t="n"/>
+      <c r="I499" s="22" t="n"/>
+      <c r="J499" s="22" t="n"/>
+    </row>
+    <row r="500" ht="20" customHeight="1">
+      <c r="A500" s="6" t="n"/>
+      <c r="B500" s="6" t="n"/>
+      <c r="C500" s="23" t="inlineStr">
         <is>
           <t>Tesis içi yol güzergâhı: 745,57 m² alan, ortalama 5,00 m genişlik -&gt; 149,11 m uzunluk</t>
         </is>
       </c>
-      <c r="D495" s="6" t="n"/>
-      <c r="E495" s="28" t="n">
+      <c r="D500" s="6" t="n"/>
+      <c r="E500" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F495" s="29" t="n">
+      <c r="F500" s="29" t="n">
         <v>5</v>
       </c>
-      <c r="G495" s="29" t="n">
+      <c r="G500" s="29" t="n">
         <v>149.11</v>
       </c>
-      <c r="H495" s="29" t="n">
+      <c r="H500" s="29" t="n">
         <v>0.35</v>
       </c>
-      <c r="I495" s="24">
-        <f>E495*F495*G495*H495</f>
-        <v/>
-      </c>
-      <c r="J495" s="6" t="n"/>
-    </row>
-    <row r="496">
-      <c r="A496" s="22" t="n"/>
-      <c r="B496" s="22" t="n"/>
-      <c r="C496" s="25" t="inlineStr">
+      <c r="I500" s="24">
+        <f>E500*F500*G500*H500</f>
+        <v/>
+      </c>
+      <c r="J500" s="6" t="n"/>
+    </row>
+    <row r="501">
+      <c r="A501" s="22" t="n"/>
+      <c r="B501" s="22" t="n"/>
+      <c r="C501" s="25" t="inlineStr">
         <is>
           <t>M02 TOPLAMI</t>
         </is>
       </c>
-      <c r="D496" s="26" t="inlineStr">
+      <c r="D501" s="26" t="inlineStr">
         <is>
           <t>m³</t>
-        </is>
-      </c>
-      <c r="E496" s="22" t="n"/>
-      <c r="F496" s="22" t="n"/>
-      <c r="G496" s="22" t="n"/>
-      <c r="H496" s="22" t="n"/>
-      <c r="I496" s="22" t="n"/>
-      <c r="J496" s="27">
-        <f>SUM(I495:I495)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="497" ht="22" customHeight="1">
-      <c r="A497" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="B497" s="20" t="inlineStr">
-        <is>
-          <t>TKDK-0091</t>
-        </is>
-      </c>
-      <c r="C497" s="8" t="inlineStr">
-        <is>
-          <t>[M46]  1,50 m yükseklikte sıcak daldırma galvanizli tel örgü ile çit yapılması</t>
-        </is>
-      </c>
-      <c r="D497" s="21" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E497" s="22" t="n"/>
-      <c r="F497" s="22" t="n"/>
-      <c r="G497" s="22" t="n"/>
-      <c r="H497" s="22" t="n"/>
-      <c r="I497" s="22" t="n"/>
-      <c r="J497" s="22" t="n"/>
-    </row>
-    <row r="498" ht="30" customHeight="1">
-      <c r="A498" s="6" t="n"/>
-      <c r="B498" s="6" t="n"/>
-      <c r="C498" s="23" t="inlineStr">
-        <is>
-          <t>Parsel 7.966,67 m²; yerleşim planındaki cephe 113,04 m, buna karşılık gelen derinlik 7.966,67/113,04 = 70,48 m; çevre 2x(113,04+70,48)</t>
-        </is>
-      </c>
-      <c r="D498" s="6" t="n"/>
-      <c r="E498" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F498" s="6" t="n"/>
-      <c r="G498" s="29" t="n">
-        <v>367.04</v>
-      </c>
-      <c r="H498" s="6" t="n"/>
-      <c r="I498" s="24">
-        <f>E498*G498</f>
-        <v/>
-      </c>
-      <c r="J498" s="6" t="n"/>
-    </row>
-    <row r="499" ht="12" customHeight="1">
-      <c r="A499" s="6" t="n"/>
-      <c r="B499" s="6" t="n"/>
-      <c r="C499" s="23" t="inlineStr">
-        <is>
-          <t>Giriş kapısı açıklığı düşülür</t>
-        </is>
-      </c>
-      <c r="D499" s="6" t="n"/>
-      <c r="E499" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F499" s="6" t="n"/>
-      <c r="G499" s="29" t="n">
-        <v>6</v>
-      </c>
-      <c r="H499" s="6" t="n"/>
-      <c r="I499" s="24">
-        <f>-E499*G499</f>
-        <v/>
-      </c>
-      <c r="J499" s="6" t="n"/>
-    </row>
-    <row r="500">
-      <c r="A500" s="22" t="n"/>
-      <c r="B500" s="22" t="n"/>
-      <c r="C500" s="25" t="inlineStr">
-        <is>
-          <t>M46 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D500" s="26" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E500" s="22" t="n"/>
-      <c r="F500" s="22" t="n"/>
-      <c r="G500" s="22" t="n"/>
-      <c r="H500" s="22" t="n"/>
-      <c r="I500" s="22" t="n"/>
-      <c r="J500" s="27">
-        <f>SUM(I498:I499)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="501" ht="22" customHeight="1">
-      <c r="A501" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="B501" s="20" t="inlineStr">
-        <is>
-          <t>43.527.1001</t>
-        </is>
-      </c>
-      <c r="C501" s="8" t="inlineStr">
-        <is>
-          <t>[M59]  ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
-        </is>
-      </c>
-      <c r="D501" s="21" t="inlineStr">
-        <is>
-          <t>m</t>
         </is>
       </c>
       <c r="E501" s="22" t="n"/>
@@ -12943,37 +12937,43 @@
       <c r="G501" s="22" t="n"/>
       <c r="H501" s="22" t="n"/>
       <c r="I501" s="22" t="n"/>
-      <c r="J501" s="22" t="n"/>
-    </row>
-    <row r="502" ht="12" customHeight="1">
-      <c r="A502" s="6" t="n"/>
-      <c r="B502" s="6" t="n"/>
-      <c r="C502" s="23" t="inlineStr">
-        <is>
-          <t>Kümes A blok servis bölümü - foseptik</t>
-        </is>
-      </c>
-      <c r="D502" s="6" t="n"/>
-      <c r="E502" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F502" s="6" t="n"/>
-      <c r="G502" s="29" t="n">
-        <v>25</v>
-      </c>
-      <c r="H502" s="6" t="n"/>
-      <c r="I502" s="24">
-        <f>E502*G502</f>
-        <v/>
-      </c>
-      <c r="J502" s="6" t="n"/>
-    </row>
-    <row r="503" ht="12" customHeight="1">
+      <c r="J501" s="27">
+        <f>SUM(I500:I500)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="502" ht="22" customHeight="1">
+      <c r="A502" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B502" s="20" t="inlineStr">
+        <is>
+          <t>TKDK-0091</t>
+        </is>
+      </c>
+      <c r="C502" s="8" t="inlineStr">
+        <is>
+          <t>[M46]  1,50 m yükseklikte sıcak daldırma galvanizli tel örgü ile çit yapılması</t>
+        </is>
+      </c>
+      <c r="D502" s="21" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E502" s="22" t="n"/>
+      <c r="F502" s="22" t="n"/>
+      <c r="G502" s="22" t="n"/>
+      <c r="H502" s="22" t="n"/>
+      <c r="I502" s="22" t="n"/>
+      <c r="J502" s="22" t="n"/>
+    </row>
+    <row r="503" ht="30" customHeight="1">
       <c r="A503" s="6" t="n"/>
       <c r="B503" s="6" t="n"/>
       <c r="C503" s="23" t="inlineStr">
         <is>
-          <t>Kümes B blok servis bölümü - foseptik</t>
+          <t>Parsel 7.966,67 m²; yerleşim planındaki cephe 113,04 m, buna karşılık gelen derinlik 7.966,67/113,04 = 70,48 m; çevre 2x(113,04+70,48)</t>
         </is>
       </c>
       <c r="D503" s="6" t="n"/>
@@ -12982,7 +12982,7 @@
       </c>
       <c r="F503" s="6" t="n"/>
       <c r="G503" s="29" t="n">
-        <v>25</v>
+        <v>367.04</v>
       </c>
       <c r="H503" s="6" t="n"/>
       <c r="I503" s="24">
@@ -12991,46 +12991,40 @@
       </c>
       <c r="J503" s="6" t="n"/>
     </row>
-    <row r="504">
-      <c r="A504" s="22" t="n"/>
-      <c r="B504" s="22" t="n"/>
-      <c r="C504" s="25" t="inlineStr">
-        <is>
-          <t>M59 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D504" s="26" t="inlineStr">
+    <row r="504" ht="12" customHeight="1">
+      <c r="A504" s="6" t="n"/>
+      <c r="B504" s="6" t="n"/>
+      <c r="C504" s="23" t="inlineStr">
+        <is>
+          <t>Giriş kapısı açıklığı düşülür</t>
+        </is>
+      </c>
+      <c r="D504" s="6" t="n"/>
+      <c r="E504" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F504" s="6" t="n"/>
+      <c r="G504" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="H504" s="6" t="n"/>
+      <c r="I504" s="24">
+        <f>-E504*G504</f>
+        <v/>
+      </c>
+      <c r="J504" s="6" t="n"/>
+    </row>
+    <row r="505">
+      <c r="A505" s="22" t="n"/>
+      <c r="B505" s="22" t="n"/>
+      <c r="C505" s="25" t="inlineStr">
+        <is>
+          <t>M46 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D505" s="26" t="inlineStr">
         <is>
           <t>m</t>
-        </is>
-      </c>
-      <c r="E504" s="22" t="n"/>
-      <c r="F504" s="22" t="n"/>
-      <c r="G504" s="22" t="n"/>
-      <c r="H504" s="22" t="n"/>
-      <c r="I504" s="22" t="n"/>
-      <c r="J504" s="27">
-        <f>SUM(I502:I503)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="505" ht="15" customHeight="1">
-      <c r="A505" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="B505" s="20" t="inlineStr">
-        <is>
-          <t>15.150.1005</t>
-        </is>
-      </c>
-      <c r="C505" s="8" t="inlineStr">
-        <is>
-          <t>[M61A]  C 25/30 hazır beton dökülmesi — betonarme rögarlar</t>
-        </is>
-      </c>
-      <c r="D505" s="21" t="inlineStr">
-        <is>
-          <t>m³</t>
         </is>
       </c>
       <c r="E505" s="22" t="n"/>
@@ -13038,102 +13032,94 @@
       <c r="G505" s="22" t="n"/>
       <c r="H505" s="22" t="n"/>
       <c r="I505" s="22" t="n"/>
-      <c r="J505" s="22" t="n"/>
-    </row>
-    <row r="506" ht="12" customHeight="1">
-      <c r="A506" s="6" t="n"/>
-      <c r="B506" s="6" t="n"/>
-      <c r="C506" s="23" t="inlineStr">
-        <is>
-          <t>Dış prizma: 0,90 x 0,90 x 0,75; 4 adet</t>
-        </is>
-      </c>
-      <c r="D506" s="6" t="n"/>
-      <c r="E506" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="F506" s="29" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G506" s="29" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H506" s="29" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="I506" s="24">
-        <f>E506*F506*G506*H506</f>
-        <v/>
-      </c>
-      <c r="J506" s="6" t="n"/>
+      <c r="J505" s="27">
+        <f>SUM(I503:I504)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="506" ht="22" customHeight="1">
+      <c r="A506" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B506" s="20" t="inlineStr">
+        <is>
+          <t>43.527.1001</t>
+        </is>
+      </c>
+      <c r="C506" s="8" t="inlineStr">
+        <is>
+          <t>[M59]  ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+        </is>
+      </c>
+      <c r="D506" s="21" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E506" s="22" t="n"/>
+      <c r="F506" s="22" t="n"/>
+      <c r="G506" s="22" t="n"/>
+      <c r="H506" s="22" t="n"/>
+      <c r="I506" s="22" t="n"/>
+      <c r="J506" s="22" t="n"/>
     </row>
     <row r="507" ht="12" customHeight="1">
       <c r="A507" s="6" t="n"/>
       <c r="B507" s="6" t="n"/>
       <c r="C507" s="23" t="inlineStr">
         <is>
-          <t>Net iç hacim düşülür: 0,60 x 0,60 x 0,60; 4 adet</t>
+          <t>Kümes A blok servis bölümü - foseptik</t>
         </is>
       </c>
       <c r="D507" s="6" t="n"/>
       <c r="E507" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="F507" s="29" t="n">
-        <v>0.6</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="F507" s="6" t="n"/>
       <c r="G507" s="29" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H507" s="29" t="n">
-        <v>0.6</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="H507" s="6" t="n"/>
       <c r="I507" s="24">
-        <f>-E507*F507*G507*H507</f>
+        <f>E507*G507</f>
         <v/>
       </c>
       <c r="J507" s="6" t="n"/>
     </row>
-    <row r="508">
-      <c r="A508" s="22" t="n"/>
-      <c r="B508" s="22" t="n"/>
-      <c r="C508" s="25" t="inlineStr">
-        <is>
-          <t>M61A TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D508" s="26" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E508" s="22" t="n"/>
-      <c r="F508" s="22" t="n"/>
-      <c r="G508" s="22" t="n"/>
-      <c r="H508" s="22" t="n"/>
-      <c r="I508" s="22" t="n"/>
-      <c r="J508" s="27">
-        <f>SUM(I506:I507)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="509" ht="22" customHeight="1">
-      <c r="A509" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="B509" s="20" t="inlineStr">
-        <is>
-          <t>15.180.1003</t>
-        </is>
-      </c>
-      <c r="C509" s="8" t="inlineStr">
-        <is>
-          <t>[M61B]  Düz yüzeyli beton ve betonarme kalıbı yapılması — betonarme rögarlar</t>
-        </is>
-      </c>
-      <c r="D509" s="21" t="inlineStr">
-        <is>
-          <t>m²</t>
+    <row r="508" ht="12" customHeight="1">
+      <c r="A508" s="6" t="n"/>
+      <c r="B508" s="6" t="n"/>
+      <c r="C508" s="23" t="inlineStr">
+        <is>
+          <t>Kümes B blok servis bölümü - foseptik</t>
+        </is>
+      </c>
+      <c r="D508" s="6" t="n"/>
+      <c r="E508" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F508" s="6" t="n"/>
+      <c r="G508" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="H508" s="6" t="n"/>
+      <c r="I508" s="24">
+        <f>E508*G508</f>
+        <v/>
+      </c>
+      <c r="J508" s="6" t="n"/>
+    </row>
+    <row r="509">
+      <c r="A509" s="22" t="n"/>
+      <c r="B509" s="22" t="n"/>
+      <c r="C509" s="25" t="inlineStr">
+        <is>
+          <t>M59 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D509" s="26" t="inlineStr">
+        <is>
+          <t>m</t>
         </is>
       </c>
       <c r="E509" s="22" t="n"/>
@@ -13141,41 +13127,43 @@
       <c r="G509" s="22" t="n"/>
       <c r="H509" s="22" t="n"/>
       <c r="I509" s="22" t="n"/>
-      <c r="J509" s="22" t="n"/>
-    </row>
-    <row r="510" ht="12" customHeight="1">
-      <c r="A510" s="6" t="n"/>
-      <c r="B510" s="6" t="n"/>
-      <c r="C510" s="23" t="inlineStr">
-        <is>
-          <t>İç yüzler: 4 yüz x 0,60 x 0,60; 4 adet</t>
-        </is>
-      </c>
-      <c r="D510" s="6" t="n"/>
-      <c r="E510" s="28" t="n">
+      <c r="J509" s="27">
+        <f>SUM(I507:I508)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="510" ht="15" customHeight="1">
+      <c r="A510" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="F510" s="29" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G510" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="H510" s="29" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I510" s="24">
-        <f>E510*F510*G510*H510</f>
-        <v/>
-      </c>
-      <c r="J510" s="6" t="n"/>
+      <c r="B510" s="20" t="inlineStr">
+        <is>
+          <t>15.150.1005</t>
+        </is>
+      </c>
+      <c r="C510" s="8" t="inlineStr">
+        <is>
+          <t>[M61A]  C 25/30 hazır beton dökülmesi — betonarme rögarlar</t>
+        </is>
+      </c>
+      <c r="D510" s="21" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E510" s="22" t="n"/>
+      <c r="F510" s="22" t="n"/>
+      <c r="G510" s="22" t="n"/>
+      <c r="H510" s="22" t="n"/>
+      <c r="I510" s="22" t="n"/>
+      <c r="J510" s="22" t="n"/>
     </row>
     <row r="511" ht="12" customHeight="1">
       <c r="A511" s="6" t="n"/>
       <c r="B511" s="6" t="n"/>
       <c r="C511" s="23" t="inlineStr">
         <is>
-          <t>Dış yüzler: 4 yüz x 0,90 x 0,60; 4 adet</t>
+          <t>Dış prizma: 0,90 x 0,90 x 0,75; 4 adet</t>
         </is>
       </c>
       <c r="D511" s="6" t="n"/>
@@ -13186,10 +13174,10 @@
         <v>0.9</v>
       </c>
       <c r="G511" s="29" t="n">
-        <v>4</v>
+        <v>0.9</v>
       </c>
       <c r="H511" s="29" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="I511" s="24">
         <f>E511*F511*G511*H511</f>
@@ -13197,46 +13185,44 @@
       </c>
       <c r="J511" s="6" t="n"/>
     </row>
-    <row r="512">
-      <c r="A512" s="22" t="n"/>
-      <c r="B512" s="22" t="n"/>
-      <c r="C512" s="25" t="inlineStr">
-        <is>
-          <t>M61B TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D512" s="26" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E512" s="22" t="n"/>
-      <c r="F512" s="22" t="n"/>
-      <c r="G512" s="22" t="n"/>
-      <c r="H512" s="22" t="n"/>
-      <c r="I512" s="22" t="n"/>
-      <c r="J512" s="27">
-        <f>SUM(I510:I511)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="513" ht="15" customHeight="1">
-      <c r="A513" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="B513" s="20" t="inlineStr">
-        <is>
-          <t>15.160.1003</t>
-        </is>
-      </c>
-      <c r="C513" s="8" t="inlineStr">
-        <is>
-          <t>[M61C]  Nervürlü betonarme çeliği ø8-ø12 — betonarme rögarlar</t>
-        </is>
-      </c>
-      <c r="D513" s="21" t="inlineStr">
-        <is>
-          <t>ton</t>
+    <row r="512" ht="12" customHeight="1">
+      <c r="A512" s="6" t="n"/>
+      <c r="B512" s="6" t="n"/>
+      <c r="C512" s="23" t="inlineStr">
+        <is>
+          <t>Net iç hacim düşülür: 0,60 x 0,60 x 0,60; 4 adet</t>
+        </is>
+      </c>
+      <c r="D512" s="6" t="n"/>
+      <c r="E512" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="F512" s="29" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G512" s="29" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H512" s="29" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I512" s="24">
+        <f>-E512*F512*G512*H512</f>
+        <v/>
+      </c>
+      <c r="J512" s="6" t="n"/>
+    </row>
+    <row r="513">
+      <c r="A513" s="22" t="n"/>
+      <c r="B513" s="22" t="n"/>
+      <c r="C513" s="25" t="inlineStr">
+        <is>
+          <t>M61A TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D513" s="26" t="inlineStr">
+        <is>
+          <t>m³</t>
         </is>
       </c>
       <c r="E513" s="22" t="n"/>
@@ -13244,114 +13230,131 @@
       <c r="G513" s="22" t="n"/>
       <c r="H513" s="22" t="n"/>
       <c r="I513" s="22" t="n"/>
-      <c r="J513" s="22" t="n"/>
-    </row>
-    <row r="514" ht="20" customHeight="1">
-      <c r="A514" s="6" t="n"/>
-      <c r="B514" s="6" t="n"/>
-      <c r="C514" s="23" t="inlineStr">
-        <is>
-          <t>Beton hacmi 1,566 m³, ortalama donatı oranı 90 kg/m³ -&gt; 140,94 kg = 0,141 ton</t>
-        </is>
-      </c>
-      <c r="D514" s="6" t="n"/>
-      <c r="E514" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F514" s="6" t="n"/>
-      <c r="G514" s="29" t="n">
-        <v>1.566</v>
-      </c>
-      <c r="H514" s="6" t="n"/>
-      <c r="I514" s="24">
-        <f>E514*G514*J514</f>
-        <v/>
-      </c>
-      <c r="J514" s="30" t="n">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="515">
-      <c r="A515" s="22" t="n"/>
-      <c r="B515" s="22" t="n"/>
-      <c r="C515" s="25" t="inlineStr">
-        <is>
-          <t>M61C TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D515" s="26" t="inlineStr">
+      <c r="J513" s="27">
+        <f>SUM(I511:I512)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="514" ht="22" customHeight="1">
+      <c r="A514" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="B514" s="20" t="inlineStr">
+        <is>
+          <t>15.180.1003</t>
+        </is>
+      </c>
+      <c r="C514" s="8" t="inlineStr">
+        <is>
+          <t>[M61B]  Düz yüzeyli beton ve betonarme kalıbı yapılması — betonarme rögarlar</t>
+        </is>
+      </c>
+      <c r="D514" s="21" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E514" s="22" t="n"/>
+      <c r="F514" s="22" t="n"/>
+      <c r="G514" s="22" t="n"/>
+      <c r="H514" s="22" t="n"/>
+      <c r="I514" s="22" t="n"/>
+      <c r="J514" s="22" t="n"/>
+    </row>
+    <row r="515" ht="12" customHeight="1">
+      <c r="A515" s="6" t="n"/>
+      <c r="B515" s="6" t="n"/>
+      <c r="C515" s="23" t="inlineStr">
+        <is>
+          <t>İç yüzler: 4 yüz x 0,60 x 0,60; 4 adet</t>
+        </is>
+      </c>
+      <c r="D515" s="6" t="n"/>
+      <c r="E515" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="F515" s="29" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G515" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="H515" s="29" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I515" s="24">
+        <f>E515*F515*G515*H515</f>
+        <v/>
+      </c>
+      <c r="J515" s="6" t="n"/>
+    </row>
+    <row r="516" ht="12" customHeight="1">
+      <c r="A516" s="6" t="n"/>
+      <c r="B516" s="6" t="n"/>
+      <c r="C516" s="23" t="inlineStr">
+        <is>
+          <t>Dış yüzler: 4 yüz x 0,90 x 0,60; 4 adet</t>
+        </is>
+      </c>
+      <c r="D516" s="6" t="n"/>
+      <c r="E516" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="F516" s="29" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G516" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="H516" s="29" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I516" s="24">
+        <f>E516*F516*G516*H516</f>
+        <v/>
+      </c>
+      <c r="J516" s="6" t="n"/>
+    </row>
+    <row r="517">
+      <c r="A517" s="22" t="n"/>
+      <c r="B517" s="22" t="n"/>
+      <c r="C517" s="25" t="inlineStr">
+        <is>
+          <t>M61B TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D517" s="26" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E517" s="22" t="n"/>
+      <c r="F517" s="22" t="n"/>
+      <c r="G517" s="22" t="n"/>
+      <c r="H517" s="22" t="n"/>
+      <c r="I517" s="22" t="n"/>
+      <c r="J517" s="27">
+        <f>SUM(I515:I516)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="518" ht="15" customHeight="1">
+      <c r="A518" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B518" s="20" t="inlineStr">
+        <is>
+          <t>15.160.1003</t>
+        </is>
+      </c>
+      <c r="C518" s="8" t="inlineStr">
+        <is>
+          <t>[M61C]  Nervürlü betonarme çeliği ø8-ø12 — betonarme rögarlar</t>
+        </is>
+      </c>
+      <c r="D518" s="21" t="inlineStr">
         <is>
           <t>ton</t>
-        </is>
-      </c>
-      <c r="E515" s="22" t="n"/>
-      <c r="F515" s="22" t="n"/>
-      <c r="G515" s="22" t="n"/>
-      <c r="H515" s="22" t="n"/>
-      <c r="I515" s="22" t="n"/>
-      <c r="J515" s="27">
-        <f>SUM(I514:I514)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="516" ht="15" customHeight="1">
-      <c r="A516" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="B516" s="20" t="inlineStr">
-        <is>
-          <t>15.560.1003</t>
-        </is>
-      </c>
-      <c r="C516" s="8" t="inlineStr">
-        <is>
-          <t>[M61D]  Betonarme kompozit rögar kapağı temini ve yerine konulması</t>
-        </is>
-      </c>
-      <c r="D516" s="21" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E516" s="22" t="n"/>
-      <c r="F516" s="22" t="n"/>
-      <c r="G516" s="22" t="n"/>
-      <c r="H516" s="22" t="n"/>
-      <c r="I516" s="22" t="n"/>
-      <c r="J516" s="22" t="n"/>
-    </row>
-    <row r="517" ht="12" customHeight="1">
-      <c r="A517" s="6" t="n"/>
-      <c r="B517" s="6" t="n"/>
-      <c r="C517" s="23" t="inlineStr">
-        <is>
-          <t>Pissu hattında 4 adet</t>
-        </is>
-      </c>
-      <c r="D517" s="6" t="n"/>
-      <c r="E517" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="F517" s="6" t="n"/>
-      <c r="G517" s="6" t="n"/>
-      <c r="H517" s="6" t="n"/>
-      <c r="I517" s="24">
-        <f>E517</f>
-        <v/>
-      </c>
-      <c r="J517" s="6" t="n"/>
-    </row>
-    <row r="518">
-      <c r="A518" s="22" t="n"/>
-      <c r="B518" s="22" t="n"/>
-      <c r="C518" s="25" t="inlineStr">
-        <is>
-          <t>M61D TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D518" s="26" t="inlineStr">
-        <is>
-          <t>ad</t>
         </is>
       </c>
       <c r="E518" s="22" t="n"/>
@@ -13359,69 +13362,71 @@
       <c r="G518" s="22" t="n"/>
       <c r="H518" s="22" t="n"/>
       <c r="I518" s="22" t="n"/>
-      <c r="J518" s="27">
-        <f>SUM(I517:I517)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="519" ht="22" customHeight="1">
-      <c r="A519" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="B519" s="20" t="inlineStr">
-        <is>
-          <t>35.100.1104</t>
-        </is>
-      </c>
-      <c r="C519" s="8" t="inlineStr">
-        <is>
-          <t>[M63]  Ana dağıtım panosu (dikili tip galvanizli sac, en az 700 mm en, 400 mm derinlik)</t>
-        </is>
-      </c>
-      <c r="D519" s="21" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E519" s="22" t="n"/>
-      <c r="F519" s="22" t="n"/>
-      <c r="G519" s="22" t="n"/>
-      <c r="H519" s="22" t="n"/>
-      <c r="I519" s="22" t="n"/>
-      <c r="J519" s="22" t="n"/>
-    </row>
-    <row r="520" ht="12" customHeight="1">
-      <c r="A520" s="6" t="n"/>
-      <c r="B520" s="6" t="n"/>
-      <c r="C520" s="23" t="inlineStr">
-        <is>
-          <t>Tesis girişinde 1 adet</t>
-        </is>
-      </c>
-      <c r="D520" s="6" t="n"/>
-      <c r="E520" s="28" t="n">
+      <c r="J518" s="22" t="n"/>
+    </row>
+    <row r="519" ht="20" customHeight="1">
+      <c r="A519" s="6" t="n"/>
+      <c r="B519" s="6" t="n"/>
+      <c r="C519" s="23" t="inlineStr">
+        <is>
+          <t>Beton hacmi 1,566 m³, ortalama donatı oranı 90 kg/m³ -&gt; 140,94 kg = 0,141 ton</t>
+        </is>
+      </c>
+      <c r="D519" s="6" t="n"/>
+      <c r="E519" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F520" s="6" t="n"/>
-      <c r="G520" s="6" t="n"/>
-      <c r="H520" s="6" t="n"/>
-      <c r="I520" s="24">
-        <f>E520*J520</f>
-        <v/>
-      </c>
-      <c r="J520" s="30" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="521">
-      <c r="A521" s="22" t="n"/>
-      <c r="B521" s="22" t="n"/>
-      <c r="C521" s="25" t="inlineStr">
-        <is>
-          <t>M63 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D521" s="26" t="inlineStr">
+      <c r="F519" s="6" t="n"/>
+      <c r="G519" s="29" t="n">
+        <v>1.566</v>
+      </c>
+      <c r="H519" s="6" t="n"/>
+      <c r="I519" s="24">
+        <f>E519*G519*J519</f>
+        <v/>
+      </c>
+      <c r="J519" s="30" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="22" t="n"/>
+      <c r="B520" s="22" t="n"/>
+      <c r="C520" s="25" t="inlineStr">
+        <is>
+          <t>M61C TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D520" s="26" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="E520" s="22" t="n"/>
+      <c r="F520" s="22" t="n"/>
+      <c r="G520" s="22" t="n"/>
+      <c r="H520" s="22" t="n"/>
+      <c r="I520" s="22" t="n"/>
+      <c r="J520" s="27">
+        <f>SUM(I519:I519)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="521" ht="15" customHeight="1">
+      <c r="A521" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="B521" s="20" t="inlineStr">
+        <is>
+          <t>15.560.1003</t>
+        </is>
+      </c>
+      <c r="C521" s="8" t="inlineStr">
+        <is>
+          <t>[M61D]  Betonarme kompozit rögar kapağı temini ve yerine konulması</t>
+        </is>
+      </c>
+      <c r="D521" s="21" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
@@ -13431,69 +13436,67 @@
       <c r="G521" s="22" t="n"/>
       <c r="H521" s="22" t="n"/>
       <c r="I521" s="22" t="n"/>
-      <c r="J521" s="27">
-        <f>SUM(I520:I520)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="522" ht="15" customHeight="1">
-      <c r="A522" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="B522" s="20" t="inlineStr">
-        <is>
-          <t>35.100.2106</t>
-        </is>
-      </c>
-      <c r="C522" s="8" t="inlineStr">
-        <is>
-          <t>[M64]  Sayaç panosu (sıva üstü galvanizli sac tablo, 0,50-0,60 m²)</t>
-        </is>
-      </c>
-      <c r="D522" s="21" t="inlineStr">
+      <c r="J521" s="22" t="n"/>
+    </row>
+    <row r="522" ht="12" customHeight="1">
+      <c r="A522" s="6" t="n"/>
+      <c r="B522" s="6" t="n"/>
+      <c r="C522" s="23" t="inlineStr">
+        <is>
+          <t>Pissu hattında 4 adet</t>
+        </is>
+      </c>
+      <c r="D522" s="6" t="n"/>
+      <c r="E522" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="F522" s="6" t="n"/>
+      <c r="G522" s="6" t="n"/>
+      <c r="H522" s="6" t="n"/>
+      <c r="I522" s="24">
+        <f>E522</f>
+        <v/>
+      </c>
+      <c r="J522" s="6" t="n"/>
+    </row>
+    <row r="523">
+      <c r="A523" s="22" t="n"/>
+      <c r="B523" s="22" t="n"/>
+      <c r="C523" s="25" t="inlineStr">
+        <is>
+          <t>M61D TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D523" s="26" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
       </c>
-      <c r="E522" s="22" t="n"/>
-      <c r="F522" s="22" t="n"/>
-      <c r="G522" s="22" t="n"/>
-      <c r="H522" s="22" t="n"/>
-      <c r="I522" s="22" t="n"/>
-      <c r="J522" s="22" t="n"/>
-    </row>
-    <row r="523" ht="12" customHeight="1">
-      <c r="A523" s="6" t="n"/>
-      <c r="B523" s="6" t="n"/>
-      <c r="C523" s="23" t="inlineStr">
-        <is>
-          <t>Tesis girişinde 1 adet</t>
-        </is>
-      </c>
-      <c r="D523" s="6" t="n"/>
-      <c r="E523" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F523" s="6" t="n"/>
-      <c r="G523" s="6" t="n"/>
-      <c r="H523" s="6" t="n"/>
-      <c r="I523" s="24">
-        <f>E523*J523</f>
-        <v/>
-      </c>
-      <c r="J523" s="30" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="524">
-      <c r="A524" s="22" t="n"/>
-      <c r="B524" s="22" t="n"/>
-      <c r="C524" s="25" t="inlineStr">
-        <is>
-          <t>M64 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D524" s="26" t="inlineStr">
+      <c r="E523" s="22" t="n"/>
+      <c r="F523" s="22" t="n"/>
+      <c r="G523" s="22" t="n"/>
+      <c r="H523" s="22" t="n"/>
+      <c r="I523" s="22" t="n"/>
+      <c r="J523" s="27">
+        <f>SUM(I522:I522)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="524" ht="22" customHeight="1">
+      <c r="A524" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="B524" s="20" t="inlineStr">
+        <is>
+          <t>35.100.1104</t>
+        </is>
+      </c>
+      <c r="C524" s="8" t="inlineStr">
+        <is>
+          <t>[M63]  Ana dağıtım panosu (dikili tip galvanizli sac, en az 700 mm en, 400 mm derinlik)</t>
+        </is>
+      </c>
+      <c r="D524" s="21" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
@@ -13503,69 +13506,69 @@
       <c r="G524" s="22" t="n"/>
       <c r="H524" s="22" t="n"/>
       <c r="I524" s="22" t="n"/>
-      <c r="J524" s="27">
-        <f>SUM(I523:I523)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="525" ht="22" customHeight="1">
-      <c r="A525" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="B525" s="20" t="inlineStr">
-        <is>
-          <t>35.135.3201</t>
-        </is>
-      </c>
-      <c r="C525" s="8" t="inlineStr">
-        <is>
-          <t>[M65]  Üç fazlı zaman tarifeli elektronik aktif sayaç, en az 5(100) A, 3x230/400 V</t>
-        </is>
-      </c>
-      <c r="D525" s="21" t="inlineStr">
+      <c r="J524" s="22" t="n"/>
+    </row>
+    <row r="525" ht="12" customHeight="1">
+      <c r="A525" s="6" t="n"/>
+      <c r="B525" s="6" t="n"/>
+      <c r="C525" s="23" t="inlineStr">
+        <is>
+          <t>Tesis girişinde 1 adet</t>
+        </is>
+      </c>
+      <c r="D525" s="6" t="n"/>
+      <c r="E525" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F525" s="6" t="n"/>
+      <c r="G525" s="6" t="n"/>
+      <c r="H525" s="6" t="n"/>
+      <c r="I525" s="24">
+        <f>E525*J525</f>
+        <v/>
+      </c>
+      <c r="J525" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="22" t="n"/>
+      <c r="B526" s="22" t="n"/>
+      <c r="C526" s="25" t="inlineStr">
+        <is>
+          <t>M63 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D526" s="26" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
       </c>
-      <c r="E525" s="22" t="n"/>
-      <c r="F525" s="22" t="n"/>
-      <c r="G525" s="22" t="n"/>
-      <c r="H525" s="22" t="n"/>
-      <c r="I525" s="22" t="n"/>
-      <c r="J525" s="22" t="n"/>
-    </row>
-    <row r="526" ht="12" customHeight="1">
-      <c r="A526" s="6" t="n"/>
-      <c r="B526" s="6" t="n"/>
-      <c r="C526" s="23" t="inlineStr">
-        <is>
-          <t>Sayaç panosu içinde 1 adet</t>
-        </is>
-      </c>
-      <c r="D526" s="6" t="n"/>
-      <c r="E526" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F526" s="6" t="n"/>
-      <c r="G526" s="6" t="n"/>
-      <c r="H526" s="6" t="n"/>
-      <c r="I526" s="24">
-        <f>E526*J526</f>
-        <v/>
-      </c>
-      <c r="J526" s="30" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="527">
-      <c r="A527" s="22" t="n"/>
-      <c r="B527" s="22" t="n"/>
-      <c r="C527" s="25" t="inlineStr">
-        <is>
-          <t>M65 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D527" s="26" t="inlineStr">
+      <c r="E526" s="22" t="n"/>
+      <c r="F526" s="22" t="n"/>
+      <c r="G526" s="22" t="n"/>
+      <c r="H526" s="22" t="n"/>
+      <c r="I526" s="22" t="n"/>
+      <c r="J526" s="27">
+        <f>SUM(I525:I525)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="527" ht="15" customHeight="1">
+      <c r="A527" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="B527" s="20" t="inlineStr">
+        <is>
+          <t>35.100.2106</t>
+        </is>
+      </c>
+      <c r="C527" s="8" t="inlineStr">
+        <is>
+          <t>[M64]  Sayaç panosu (sıva üstü galvanizli sac tablo, 0,50-0,60 m²)</t>
+        </is>
+      </c>
+      <c r="D527" s="21" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
@@ -13575,69 +13578,69 @@
       <c r="G527" s="22" t="n"/>
       <c r="H527" s="22" t="n"/>
       <c r="I527" s="22" t="n"/>
-      <c r="J527" s="27">
-        <f>SUM(I526:I526)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="528" ht="22" customHeight="1">
-      <c r="A528" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="B528" s="20" t="inlineStr">
-        <is>
-          <t>35.110.1104</t>
-        </is>
-      </c>
-      <c r="C528" s="8" t="inlineStr">
-        <is>
-          <t>[M66]  Termik-manyetik kompakt şalter 3x160 A, Icu 35 kA — ana giriş</t>
-        </is>
-      </c>
-      <c r="D528" s="21" t="inlineStr">
+      <c r="J527" s="22" t="n"/>
+    </row>
+    <row r="528" ht="12" customHeight="1">
+      <c r="A528" s="6" t="n"/>
+      <c r="B528" s="6" t="n"/>
+      <c r="C528" s="23" t="inlineStr">
+        <is>
+          <t>Tesis girişinde 1 adet</t>
+        </is>
+      </c>
+      <c r="D528" s="6" t="n"/>
+      <c r="E528" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F528" s="6" t="n"/>
+      <c r="G528" s="6" t="n"/>
+      <c r="H528" s="6" t="n"/>
+      <c r="I528" s="24">
+        <f>E528*J528</f>
+        <v/>
+      </c>
+      <c r="J528" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="22" t="n"/>
+      <c r="B529" s="22" t="n"/>
+      <c r="C529" s="25" t="inlineStr">
+        <is>
+          <t>M64 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D529" s="26" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
       </c>
-      <c r="E528" s="22" t="n"/>
-      <c r="F528" s="22" t="n"/>
-      <c r="G528" s="22" t="n"/>
-      <c r="H528" s="22" t="n"/>
-      <c r="I528" s="22" t="n"/>
-      <c r="J528" s="22" t="n"/>
-    </row>
-    <row r="529" ht="12" customHeight="1">
-      <c r="A529" s="6" t="n"/>
-      <c r="B529" s="6" t="n"/>
-      <c r="C529" s="23" t="inlineStr">
-        <is>
-          <t>Ana dağıtım panosu girişi</t>
-        </is>
-      </c>
-      <c r="D529" s="6" t="n"/>
-      <c r="E529" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F529" s="6" t="n"/>
-      <c r="G529" s="6" t="n"/>
-      <c r="H529" s="6" t="n"/>
-      <c r="I529" s="24">
-        <f>E529*J529</f>
-        <v/>
-      </c>
-      <c r="J529" s="30" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="530">
-      <c r="A530" s="22" t="n"/>
-      <c r="B530" s="22" t="n"/>
-      <c r="C530" s="25" t="inlineStr">
-        <is>
-          <t>M66 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D530" s="26" t="inlineStr">
+      <c r="E529" s="22" t="n"/>
+      <c r="F529" s="22" t="n"/>
+      <c r="G529" s="22" t="n"/>
+      <c r="H529" s="22" t="n"/>
+      <c r="I529" s="22" t="n"/>
+      <c r="J529" s="27">
+        <f>SUM(I528:I528)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="530" ht="22" customHeight="1">
+      <c r="A530" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="B530" s="20" t="inlineStr">
+        <is>
+          <t>35.135.3201</t>
+        </is>
+      </c>
+      <c r="C530" s="8" t="inlineStr">
+        <is>
+          <t>[M65]  Üç fazlı zaman tarifeli elektronik aktif sayaç, en az 5(100) A, 3x230/400 V</t>
+        </is>
+      </c>
+      <c r="D530" s="21" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
@@ -13647,69 +13650,69 @@
       <c r="G530" s="22" t="n"/>
       <c r="H530" s="22" t="n"/>
       <c r="I530" s="22" t="n"/>
-      <c r="J530" s="27">
-        <f>SUM(I529:I529)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="531" ht="15" customHeight="1">
-      <c r="A531" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="B531" s="20" t="inlineStr">
-        <is>
-          <t>35.115.1003</t>
-        </is>
-      </c>
-      <c r="C531" s="8" t="inlineStr">
-        <is>
-          <t>[M69]  Kaçak akım koruma şalteri 2x63 A, 30 mA</t>
-        </is>
-      </c>
-      <c r="D531" s="21" t="inlineStr">
+      <c r="J530" s="22" t="n"/>
+    </row>
+    <row r="531" ht="12" customHeight="1">
+      <c r="A531" s="6" t="n"/>
+      <c r="B531" s="6" t="n"/>
+      <c r="C531" s="23" t="inlineStr">
+        <is>
+          <t>Sayaç panosu içinde 1 adet</t>
+        </is>
+      </c>
+      <c r="D531" s="6" t="n"/>
+      <c r="E531" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F531" s="6" t="n"/>
+      <c r="G531" s="6" t="n"/>
+      <c r="H531" s="6" t="n"/>
+      <c r="I531" s="24">
+        <f>E531*J531</f>
+        <v/>
+      </c>
+      <c r="J531" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="22" t="n"/>
+      <c r="B532" s="22" t="n"/>
+      <c r="C532" s="25" t="inlineStr">
+        <is>
+          <t>M65 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D532" s="26" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
       </c>
-      <c r="E531" s="22" t="n"/>
-      <c r="F531" s="22" t="n"/>
-      <c r="G531" s="22" t="n"/>
-      <c r="H531" s="22" t="n"/>
-      <c r="I531" s="22" t="n"/>
-      <c r="J531" s="22" t="n"/>
-    </row>
-    <row r="532" ht="12" customHeight="1">
-      <c r="A532" s="6" t="n"/>
-      <c r="B532" s="6" t="n"/>
-      <c r="C532" s="23" t="inlineStr">
-        <is>
-          <t>Ana pano ve sayaç panosunda</t>
-        </is>
-      </c>
-      <c r="D532" s="6" t="n"/>
-      <c r="E532" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F532" s="6" t="n"/>
-      <c r="G532" s="6" t="n"/>
-      <c r="H532" s="6" t="n"/>
-      <c r="I532" s="24">
-        <f>E532*J532</f>
-        <v/>
-      </c>
-      <c r="J532" s="30" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="533">
-      <c r="A533" s="22" t="n"/>
-      <c r="B533" s="22" t="n"/>
-      <c r="C533" s="25" t="inlineStr">
-        <is>
-          <t>M69 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D533" s="26" t="inlineStr">
+      <c r="E532" s="22" t="n"/>
+      <c r="F532" s="22" t="n"/>
+      <c r="G532" s="22" t="n"/>
+      <c r="H532" s="22" t="n"/>
+      <c r="I532" s="22" t="n"/>
+      <c r="J532" s="27">
+        <f>SUM(I531:I531)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="533" ht="22" customHeight="1">
+      <c r="A533" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="B533" s="20" t="inlineStr">
+        <is>
+          <t>35.110.1104</t>
+        </is>
+      </c>
+      <c r="C533" s="8" t="inlineStr">
+        <is>
+          <t>[M66]  Termik-manyetik kompakt şalter 3x160 A, Icu 35 kA — ana giriş</t>
+        </is>
+      </c>
+      <c r="D533" s="21" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
@@ -13719,71 +13722,71 @@
       <c r="G533" s="22" t="n"/>
       <c r="H533" s="22" t="n"/>
       <c r="I533" s="22" t="n"/>
-      <c r="J533" s="27">
-        <f>SUM(I532:I532)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="534" ht="22" customHeight="1">
-      <c r="A534" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="B534" s="20" t="inlineStr">
-        <is>
-          <t>35.140.3105</t>
-        </is>
-      </c>
-      <c r="C534" s="8" t="inlineStr">
-        <is>
-          <t>[M70]  YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x35 mm²</t>
-        </is>
-      </c>
-      <c r="D534" s="21" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E534" s="22" t="n"/>
-      <c r="F534" s="22" t="n"/>
-      <c r="G534" s="22" t="n"/>
-      <c r="H534" s="22" t="n"/>
-      <c r="I534" s="22" t="n"/>
-      <c r="J534" s="22" t="n"/>
-    </row>
-    <row r="535" ht="12" customHeight="1">
-      <c r="A535" s="6" t="n"/>
-      <c r="B535" s="6" t="n"/>
-      <c r="C535" s="23" t="inlineStr">
-        <is>
-          <t>Şebeke bağlantı noktası - ana dağıtım panosu</t>
-        </is>
-      </c>
-      <c r="D535" s="6" t="n"/>
-      <c r="E535" s="28" t="n">
+      <c r="J533" s="22" t="n"/>
+    </row>
+    <row r="534" ht="12" customHeight="1">
+      <c r="A534" s="6" t="n"/>
+      <c r="B534" s="6" t="n"/>
+      <c r="C534" s="23" t="inlineStr">
+        <is>
+          <t>Ana dağıtım panosu girişi</t>
+        </is>
+      </c>
+      <c r="D534" s="6" t="n"/>
+      <c r="E534" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F535" s="6" t="n"/>
-      <c r="G535" s="6" t="n"/>
-      <c r="H535" s="6" t="n"/>
-      <c r="I535" s="24">
-        <f>E535*J535</f>
-        <v/>
-      </c>
-      <c r="J535" s="30" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="536">
-      <c r="A536" s="22" t="n"/>
-      <c r="B536" s="22" t="n"/>
-      <c r="C536" s="25" t="inlineStr">
-        <is>
-          <t>M70 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D536" s="26" t="inlineStr">
-        <is>
-          <t>m</t>
+      <c r="F534" s="6" t="n"/>
+      <c r="G534" s="6" t="n"/>
+      <c r="H534" s="6" t="n"/>
+      <c r="I534" s="24">
+        <f>E534*J534</f>
+        <v/>
+      </c>
+      <c r="J534" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="22" t="n"/>
+      <c r="B535" s="22" t="n"/>
+      <c r="C535" s="25" t="inlineStr">
+        <is>
+          <t>M66 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D535" s="26" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="E535" s="22" t="n"/>
+      <c r="F535" s="22" t="n"/>
+      <c r="G535" s="22" t="n"/>
+      <c r="H535" s="22" t="n"/>
+      <c r="I535" s="22" t="n"/>
+      <c r="J535" s="27">
+        <f>SUM(I534:I534)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="536" ht="15" customHeight="1">
+      <c r="A536" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="B536" s="20" t="inlineStr">
+        <is>
+          <t>35.115.1003</t>
+        </is>
+      </c>
+      <c r="C536" s="8" t="inlineStr">
+        <is>
+          <t>[M69]  Kaçak akım koruma şalteri 2x63 A, 30 mA</t>
+        </is>
+      </c>
+      <c r="D536" s="21" t="inlineStr">
+        <is>
+          <t>ad</t>
         </is>
       </c>
       <c r="E536" s="22" t="n"/>
@@ -13791,69 +13794,69 @@
       <c r="G536" s="22" t="n"/>
       <c r="H536" s="22" t="n"/>
       <c r="I536" s="22" t="n"/>
-      <c r="J536" s="27">
-        <f>SUM(I535:I535)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="537" ht="22" customHeight="1">
-      <c r="A537" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="B537" s="20" t="inlineStr">
-        <is>
-          <t>35.140.3101</t>
-        </is>
-      </c>
-      <c r="C537" s="8" t="inlineStr">
-        <is>
-          <t>[M72]  YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x6 mm²</t>
-        </is>
-      </c>
-      <c r="D537" s="21" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E537" s="22" t="n"/>
-      <c r="F537" s="22" t="n"/>
-      <c r="G537" s="22" t="n"/>
-      <c r="H537" s="22" t="n"/>
-      <c r="I537" s="22" t="n"/>
-      <c r="J537" s="22" t="n"/>
-    </row>
-    <row r="538" ht="12" customHeight="1">
-      <c r="A538" s="6" t="n"/>
-      <c r="B538" s="6" t="n"/>
-      <c r="C538" s="23" t="inlineStr">
-        <is>
-          <t>Saha aydınlatma direkleri besleme hattı</t>
-        </is>
-      </c>
-      <c r="D538" s="6" t="n"/>
-      <c r="E538" s="28" t="n">
+      <c r="J536" s="22" t="n"/>
+    </row>
+    <row r="537" ht="12" customHeight="1">
+      <c r="A537" s="6" t="n"/>
+      <c r="B537" s="6" t="n"/>
+      <c r="C537" s="23" t="inlineStr">
+        <is>
+          <t>Ana pano ve sayaç panosunda</t>
+        </is>
+      </c>
+      <c r="D537" s="6" t="n"/>
+      <c r="E537" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F538" s="6" t="n"/>
-      <c r="G538" s="6" t="n"/>
-      <c r="H538" s="6" t="n"/>
-      <c r="I538" s="24">
-        <f>E538*J538</f>
-        <v/>
-      </c>
-      <c r="J538" s="30" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="539">
-      <c r="A539" s="22" t="n"/>
-      <c r="B539" s="22" t="n"/>
-      <c r="C539" s="25" t="inlineStr">
-        <is>
-          <t>M72 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D539" s="26" t="inlineStr">
+      <c r="F537" s="6" t="n"/>
+      <c r="G537" s="6" t="n"/>
+      <c r="H537" s="6" t="n"/>
+      <c r="I537" s="24">
+        <f>E537*J537</f>
+        <v/>
+      </c>
+      <c r="J537" s="30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="22" t="n"/>
+      <c r="B538" s="22" t="n"/>
+      <c r="C538" s="25" t="inlineStr">
+        <is>
+          <t>M69 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D538" s="26" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="E538" s="22" t="n"/>
+      <c r="F538" s="22" t="n"/>
+      <c r="G538" s="22" t="n"/>
+      <c r="H538" s="22" t="n"/>
+      <c r="I538" s="22" t="n"/>
+      <c r="J538" s="27">
+        <f>SUM(I537:I537)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="539" ht="22" customHeight="1">
+      <c r="A539" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="B539" s="20" t="inlineStr">
+        <is>
+          <t>35.140.3105</t>
+        </is>
+      </c>
+      <c r="C539" s="8" t="inlineStr">
+        <is>
+          <t>[M70]  YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x35 mm²</t>
+        </is>
+      </c>
+      <c r="D539" s="21" t="inlineStr">
         <is>
           <t>m</t>
         </is>
@@ -13863,71 +13866,71 @@
       <c r="G539" s="22" t="n"/>
       <c r="H539" s="22" t="n"/>
       <c r="I539" s="22" t="n"/>
-      <c r="J539" s="27">
-        <f>SUM(I538:I538)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="540" ht="22" customHeight="1">
-      <c r="A540" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="B540" s="20" t="inlineStr">
-        <is>
-          <t>35.172.1706</t>
-        </is>
-      </c>
-      <c r="C540" s="8" t="inlineStr">
-        <is>
-          <t>[M82]  Aydınlatma direği — taban çapı en az 80 mm, yükseklik en az 4,00 m</t>
-        </is>
-      </c>
-      <c r="D540" s="21" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E540" s="22" t="n"/>
-      <c r="F540" s="22" t="n"/>
-      <c r="G540" s="22" t="n"/>
-      <c r="H540" s="22" t="n"/>
-      <c r="I540" s="22" t="n"/>
-      <c r="J540" s="22" t="n"/>
-    </row>
-    <row r="541" ht="12" customHeight="1">
-      <c r="A541" s="6" t="n"/>
-      <c r="B541" s="6" t="n"/>
-      <c r="C541" s="23" t="inlineStr">
-        <is>
-          <t>Tesis içi yol ve saha aydınlatması</t>
-        </is>
-      </c>
-      <c r="D541" s="6" t="n"/>
-      <c r="E541" s="28" t="n">
+      <c r="J539" s="22" t="n"/>
+    </row>
+    <row r="540" ht="12" customHeight="1">
+      <c r="A540" s="6" t="n"/>
+      <c r="B540" s="6" t="n"/>
+      <c r="C540" s="23" t="inlineStr">
+        <is>
+          <t>Şebeke bağlantı noktası - ana dağıtım panosu</t>
+        </is>
+      </c>
+      <c r="D540" s="6" t="n"/>
+      <c r="E540" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F541" s="6" t="n"/>
-      <c r="G541" s="6" t="n"/>
-      <c r="H541" s="6" t="n"/>
-      <c r="I541" s="24">
-        <f>E541*J541</f>
-        <v/>
-      </c>
-      <c r="J541" s="30" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="542">
-      <c r="A542" s="22" t="n"/>
-      <c r="B542" s="22" t="n"/>
-      <c r="C542" s="25" t="inlineStr">
-        <is>
-          <t>M82 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D542" s="26" t="inlineStr">
-        <is>
-          <t>ad</t>
+      <c r="F540" s="6" t="n"/>
+      <c r="G540" s="6" t="n"/>
+      <c r="H540" s="6" t="n"/>
+      <c r="I540" s="24">
+        <f>E540*J540</f>
+        <v/>
+      </c>
+      <c r="J540" s="30" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="22" t="n"/>
+      <c r="B541" s="22" t="n"/>
+      <c r="C541" s="25" t="inlineStr">
+        <is>
+          <t>M70 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D541" s="26" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E541" s="22" t="n"/>
+      <c r="F541" s="22" t="n"/>
+      <c r="G541" s="22" t="n"/>
+      <c r="H541" s="22" t="n"/>
+      <c r="I541" s="22" t="n"/>
+      <c r="J541" s="27">
+        <f>SUM(I540:I540)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="542" ht="22" customHeight="1">
+      <c r="A542" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="B542" s="20" t="inlineStr">
+        <is>
+          <t>35.140.3101</t>
+        </is>
+      </c>
+      <c r="C542" s="8" t="inlineStr">
+        <is>
+          <t>[M72]  YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x6 mm²</t>
+        </is>
+      </c>
+      <c r="D542" s="21" t="inlineStr">
+        <is>
+          <t>m</t>
         </is>
       </c>
       <c r="E542" s="22" t="n"/>
@@ -13935,69 +13938,69 @@
       <c r="G542" s="22" t="n"/>
       <c r="H542" s="22" t="n"/>
       <c r="I542" s="22" t="n"/>
-      <c r="J542" s="27">
-        <f>SUM(I541:I541)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="543" ht="15" customHeight="1">
-      <c r="A543" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="B543" s="20" t="inlineStr">
-        <is>
-          <t>35.170.4002</t>
-        </is>
-      </c>
-      <c r="C543" s="8" t="inlineStr">
-        <is>
-          <t>[M83]  LED projektör, ışık akısı en az 5100 lm</t>
-        </is>
-      </c>
-      <c r="D543" s="21" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E543" s="22" t="n"/>
-      <c r="F543" s="22" t="n"/>
-      <c r="G543" s="22" t="n"/>
-      <c r="H543" s="22" t="n"/>
-      <c r="I543" s="22" t="n"/>
-      <c r="J543" s="22" t="n"/>
-    </row>
-    <row r="544" ht="12" customHeight="1">
-      <c r="A544" s="6" t="n"/>
-      <c r="B544" s="6" t="n"/>
-      <c r="C544" s="23" t="inlineStr">
-        <is>
-          <t>Aydınlatma direği başına 1 adet</t>
-        </is>
-      </c>
-      <c r="D544" s="6" t="n"/>
-      <c r="E544" s="28" t="n">
+      <c r="J542" s="22" t="n"/>
+    </row>
+    <row r="543" ht="12" customHeight="1">
+      <c r="A543" s="6" t="n"/>
+      <c r="B543" s="6" t="n"/>
+      <c r="C543" s="23" t="inlineStr">
+        <is>
+          <t>Saha aydınlatma direkleri besleme hattı</t>
+        </is>
+      </c>
+      <c r="D543" s="6" t="n"/>
+      <c r="E543" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F544" s="6" t="n"/>
-      <c r="G544" s="6" t="n"/>
-      <c r="H544" s="6" t="n"/>
-      <c r="I544" s="24">
-        <f>E544*J544</f>
-        <v/>
-      </c>
-      <c r="J544" s="30" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="545">
-      <c r="A545" s="22" t="n"/>
-      <c r="B545" s="22" t="n"/>
-      <c r="C545" s="25" t="inlineStr">
-        <is>
-          <t>M83 TOPLAMI</t>
-        </is>
-      </c>
-      <c r="D545" s="26" t="inlineStr">
+      <c r="F543" s="6" t="n"/>
+      <c r="G543" s="6" t="n"/>
+      <c r="H543" s="6" t="n"/>
+      <c r="I543" s="24">
+        <f>E543*J543</f>
+        <v/>
+      </c>
+      <c r="J543" s="30" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="22" t="n"/>
+      <c r="B544" s="22" t="n"/>
+      <c r="C544" s="25" t="inlineStr">
+        <is>
+          <t>M72 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D544" s="26" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E544" s="22" t="n"/>
+      <c r="F544" s="22" t="n"/>
+      <c r="G544" s="22" t="n"/>
+      <c r="H544" s="22" t="n"/>
+      <c r="I544" s="22" t="n"/>
+      <c r="J544" s="27">
+        <f>SUM(I543:I543)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="545" ht="22" customHeight="1">
+      <c r="A545" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="B545" s="20" t="inlineStr">
+        <is>
+          <t>35.172.1706</t>
+        </is>
+      </c>
+      <c r="C545" s="8" t="inlineStr">
+        <is>
+          <t>[M82]  Aydınlatma direği — taban çapı en az 80 mm, yükseklik en az 4,00 m</t>
+        </is>
+      </c>
+      <c r="D545" s="21" t="inlineStr">
         <is>
           <t>ad</t>
         </is>
@@ -14007,50 +14010,165 @@
       <c r="G545" s="22" t="n"/>
       <c r="H545" s="22" t="n"/>
       <c r="I545" s="22" t="n"/>
-      <c r="J545" s="27">
-        <f>SUM(I544:I544)</f>
-        <v/>
+      <c r="J545" s="22" t="n"/>
+    </row>
+    <row r="546" ht="12" customHeight="1">
+      <c r="A546" s="6" t="n"/>
+      <c r="B546" s="6" t="n"/>
+      <c r="C546" s="23" t="inlineStr">
+        <is>
+          <t>Tesis içi yol ve saha aydınlatması</t>
+        </is>
+      </c>
+      <c r="D546" s="6" t="n"/>
+      <c r="E546" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F546" s="6" t="n"/>
+      <c r="G546" s="6" t="n"/>
+      <c r="H546" s="6" t="n"/>
+      <c r="I546" s="24">
+        <f>E546*J546</f>
+        <v/>
+      </c>
+      <c r="J546" s="30" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="547">
-      <c r="A547" s="16" t="inlineStr">
+      <c r="A547" s="22" t="n"/>
+      <c r="B547" s="22" t="n"/>
+      <c r="C547" s="25" t="inlineStr">
+        <is>
+          <t>M82 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D547" s="26" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="E547" s="22" t="n"/>
+      <c r="F547" s="22" t="n"/>
+      <c r="G547" s="22" t="n"/>
+      <c r="H547" s="22" t="n"/>
+      <c r="I547" s="22" t="n"/>
+      <c r="J547" s="27">
+        <f>SUM(I546:I546)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="548" ht="15" customHeight="1">
+      <c r="A548" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="B548" s="20" t="inlineStr">
+        <is>
+          <t>35.170.4002</t>
+        </is>
+      </c>
+      <c r="C548" s="8" t="inlineStr">
+        <is>
+          <t>[M83]  LED projektör, ışık akısı en az 5100 lm</t>
+        </is>
+      </c>
+      <c r="D548" s="21" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="E548" s="22" t="n"/>
+      <c r="F548" s="22" t="n"/>
+      <c r="G548" s="22" t="n"/>
+      <c r="H548" s="22" t="n"/>
+      <c r="I548" s="22" t="n"/>
+      <c r="J548" s="22" t="n"/>
+    </row>
+    <row r="549" ht="12" customHeight="1">
+      <c r="A549" s="6" t="n"/>
+      <c r="B549" s="6" t="n"/>
+      <c r="C549" s="23" t="inlineStr">
+        <is>
+          <t>Aydınlatma direği başına 1 adet</t>
+        </is>
+      </c>
+      <c r="D549" s="6" t="n"/>
+      <c r="E549" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F549" s="6" t="n"/>
+      <c r="G549" s="6" t="n"/>
+      <c r="H549" s="6" t="n"/>
+      <c r="I549" s="24">
+        <f>E549*J549</f>
+        <v/>
+      </c>
+      <c r="J549" s="30" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="22" t="n"/>
+      <c r="B550" s="22" t="n"/>
+      <c r="C550" s="25" t="inlineStr">
+        <is>
+          <t>M83 TOPLAMI</t>
+        </is>
+      </c>
+      <c r="D550" s="26" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="E550" s="22" t="n"/>
+      <c r="F550" s="22" t="n"/>
+      <c r="G550" s="22" t="n"/>
+      <c r="H550" s="22" t="n"/>
+      <c r="I550" s="22" t="n"/>
+      <c r="J550" s="27">
+        <f>SUM(I549:I549)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="16" t="inlineStr">
         <is>
           <t>AÇIKLAMALAR</t>
         </is>
       </c>
-      <c r="B547" s="40" t="n"/>
-      <c r="C547" s="40" t="n"/>
-      <c r="D547" s="40" t="n"/>
-      <c r="E547" s="40" t="n"/>
-      <c r="F547" s="40" t="n"/>
-      <c r="G547" s="40" t="n"/>
-      <c r="H547" s="40" t="n"/>
-      <c r="I547" s="40" t="n"/>
-      <c r="J547" s="41" t="n"/>
-    </row>
-    <row r="548" ht="13" customHeight="1">
-      <c r="A548" s="17" t="inlineStr">
+      <c r="B552" s="40" t="n"/>
+      <c r="C552" s="40" t="n"/>
+      <c r="D552" s="40" t="n"/>
+      <c r="E552" s="40" t="n"/>
+      <c r="F552" s="40" t="n"/>
+      <c r="G552" s="40" t="n"/>
+      <c r="H552" s="40" t="n"/>
+      <c r="I552" s="40" t="n"/>
+      <c r="J552" s="41" t="n"/>
+    </row>
+    <row r="553" ht="13" customHeight="1">
+      <c r="A553" s="17" t="inlineStr">
         <is>
           <t>•  Miktar sütunundaki her formül yalnızca o satırdaki ölçü hücrelerini çarpar; hiçbir sayı formülün içine gömülmemiştir.</t>
         </is>
       </c>
     </row>
-    <row r="549" ht="13" customHeight="1">
-      <c r="A549" s="17" t="inlineStr">
+    <row r="554" ht="13" customHeight="1">
+      <c r="A554" s="17" t="inlineStr">
         <is>
           <t>•  Son sütundaki katsayı, birim ağırlık (kg/m², kg/m³, ton/m²), bindirme payı, üçgen alan çarpanı (0,50) veya adet çarpanıdır.</t>
         </is>
       </c>
     </row>
-    <row r="550" ht="22" customHeight="1">
-      <c r="A550" s="17" t="inlineStr">
+    <row r="555" ht="22" customHeight="1">
+      <c r="A555" s="17" t="inlineStr">
         <is>
           <t>•  Ölçüler mimari ve betonarme paftalardan alınmıştır; kümes temellerinin beton, kalıp ve donatı miktarları doğrudan betonarme paftasındaki METRAJ tablosundandır.</t>
         </is>
       </c>
     </row>
-    <row r="551" ht="13" customHeight="1">
-      <c r="A551" s="17" t="inlineStr">
+    <row r="556" ht="13" customHeight="1">
+      <c r="A556" s="17" t="inlineStr">
         <is>
           <t>•  (-) işaretli satırlar minha edilen (düşülen) miktarlardır.</t>
         </is>
@@ -14058,22 +14176,22 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A550:J550"/>
+    <mergeCell ref="A450:J450"/>
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A497:J497"/>
     <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A552:J552"/>
+    <mergeCell ref="A361:J361"/>
     <mergeCell ref="A415:J415"/>
-    <mergeCell ref="A361:J361"/>
-    <mergeCell ref="A549:J549"/>
-    <mergeCell ref="A492:J492"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A427:J427"/>
-    <mergeCell ref="A548:J548"/>
-    <mergeCell ref="A551:J551"/>
+    <mergeCell ref="A556:J556"/>
+    <mergeCell ref="A473:J473"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A468:J468"/>
-    <mergeCell ref="A547:J547"/>
+    <mergeCell ref="A553:J553"/>
+    <mergeCell ref="A555:J555"/>
     <mergeCell ref="A183:J183"/>
-    <mergeCell ref="A445:J445"/>
+    <mergeCell ref="A554:J554"/>
     <mergeCell ref="A392:J392"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Yayın: metraj cetveli yapı bazında ayrı nüshalar (METRAJ-YAPI-BAZINDA)
Dokuz yapı için ayrı PDF ve Word; toplu nüsha yerinde. Türkçe büyük harf
düzeltmesi yapı bantlarına işlendi. 91 -> 109 belge.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/03_METRAJ_CETVELI.xlsx
+++ b/belgeler/03_METRAJ_CETVELI.xlsx
@@ -10805,7 +10805,7 @@
     <row r="415" ht="20" customHeight="1">
       <c r="A415" s="18" t="inlineStr">
         <is>
-          <t>Yapı/Bina Adı: FOSEPTIK</t>
+          <t>Yapı/Bina Adı: FOSEPTİK</t>
         </is>
       </c>
     </row>
@@ -11086,7 +11086,7 @@
     <row r="427" ht="20" customHeight="1">
       <c r="A427" s="18" t="inlineStr">
         <is>
-          <t>Yapı/Bina Adı: YEM SILOSU BETONARME KAIDELERI</t>
+          <t>Yapı/Bina Adı: YEM SİLOSU BETONARME KAİDELERİ</t>
         </is>
       </c>
     </row>
@@ -12810,7 +12810,7 @@
     <row r="497" ht="20" customHeight="1">
       <c r="A497" s="18" t="inlineStr">
         <is>
-          <t>Yapı/Bina Adı: ÇEVRE DÜZENLEMESI VE SAHA ALTYAPISI</t>
+          <t>Yapı/Bina Adı: ÇEVRE DÜZENLEMESİ VE SAHA ALTYAPISI</t>
         </is>
       </c>
     </row>

</xml_diff>